<commit_message>
feat(mesa v3): COMENTARIO en una línea sin desbordar — wrap + altura fija 18
El texto largo queda recortado en su celda (se ve completo al hacer click,
en la barra de fórmulas) en vez de invadir CONCEPTO/CATEGORIA. Aplicado al
template compartido y a las 7 mesas del ciclo julio.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/4_pagos/efectivo/inputs/mesa_2.xlsx
+++ b/4_pagos/efectivo/inputs/mesa_2.xlsx
@@ -228,7 +228,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -273,6 +273,9 @@
     </xf>
     <xf numFmtId="0" fontId="13" fillId="7" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -639,7 +642,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K25"/>
+  <dimension ref="A1:K500"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col width="20" customWidth="1" style="12" min="1" max="1"/>
@@ -791,7 +794,7 @@
       <c r="I3" s="8" t="n"/>
       <c r="J3" s="8" t="n"/>
     </row>
-    <row r="4">
+    <row r="4" ht="18" customHeight="1" s="12">
       <c r="A4" t="inlineStr">
         <is>
           <t>Yreald Romero</t>
@@ -817,8 +820,9 @@
       <c r="G4" t="n">
         <v>0</v>
       </c>
-    </row>
-    <row r="5">
+      <c r="I4" s="19" t="n"/>
+    </row>
+    <row r="5" ht="18" customHeight="1" s="12">
       <c r="A5" t="inlineStr">
         <is>
           <t>Yreald Romero</t>
@@ -844,8 +848,9 @@
       <c r="G5" t="n">
         <v>0</v>
       </c>
-    </row>
-    <row r="6">
+      <c r="I5" s="19" t="n"/>
+    </row>
+    <row r="6" ht="18" customHeight="1" s="12">
       <c r="A6" t="inlineStr">
         <is>
           <t>Yreald Romero</t>
@@ -871,8 +876,9 @@
       <c r="G6" t="n">
         <v>0</v>
       </c>
-    </row>
-    <row r="7">
+      <c r="I6" s="19" t="n"/>
+    </row>
+    <row r="7" ht="18" customHeight="1" s="12">
       <c r="A7" t="inlineStr">
         <is>
           <t>Yreald Romero</t>
@@ -898,8 +904,9 @@
       <c r="G7" t="n">
         <v>0</v>
       </c>
-    </row>
-    <row r="8">
+      <c r="I7" s="19" t="n"/>
+    </row>
+    <row r="8" ht="18" customHeight="1" s="12">
       <c r="A8" t="inlineStr">
         <is>
           <t>Yreald Romero</t>
@@ -925,8 +932,9 @@
       <c r="G8" t="n">
         <v>0</v>
       </c>
-    </row>
-    <row r="9">
+      <c r="I8" s="19" t="n"/>
+    </row>
+    <row r="9" ht="18" customHeight="1" s="12">
       <c r="A9" t="inlineStr">
         <is>
           <t>Yreald Romero</t>
@@ -952,8 +960,9 @@
       <c r="G9" t="n">
         <v>0</v>
       </c>
-    </row>
-    <row r="10">
+      <c r="I9" s="19" t="n"/>
+    </row>
+    <row r="10" ht="18" customHeight="1" s="12">
       <c r="A10" t="inlineStr">
         <is>
           <t>Yreald Romero</t>
@@ -979,8 +988,9 @@
       <c r="G10" t="n">
         <v>0</v>
       </c>
-    </row>
-    <row r="11">
+      <c r="I10" s="19" t="n"/>
+    </row>
+    <row r="11" ht="18" customHeight="1" s="12">
       <c r="A11" t="inlineStr">
         <is>
           <t>Yreald Romero</t>
@@ -1006,8 +1016,9 @@
       <c r="G11" t="n">
         <v>0</v>
       </c>
-    </row>
-    <row r="12">
+      <c r="I11" s="19" t="n"/>
+    </row>
+    <row r="12" ht="18" customHeight="1" s="12">
       <c r="A12" t="inlineStr">
         <is>
           <t>Yreald Romero</t>
@@ -1033,8 +1044,9 @@
       <c r="G12" t="n">
         <v>0</v>
       </c>
-    </row>
-    <row r="13">
+      <c r="I12" s="19" t="n"/>
+    </row>
+    <row r="13" ht="18" customHeight="1" s="12">
       <c r="A13" t="inlineStr">
         <is>
           <t>Yreald Romero</t>
@@ -1060,8 +1072,9 @@
       <c r="G13" t="n">
         <v>0</v>
       </c>
-    </row>
-    <row r="14">
+      <c r="I13" s="19" t="n"/>
+    </row>
+    <row r="14" ht="18" customHeight="1" s="12">
       <c r="A14" t="inlineStr">
         <is>
           <t>Yreald Romero</t>
@@ -1087,8 +1100,9 @@
       <c r="G14" t="n">
         <v>0</v>
       </c>
-    </row>
-    <row r="15">
+      <c r="I14" s="19" t="n"/>
+    </row>
+    <row r="15" ht="18" customHeight="1" s="12">
       <c r="A15" t="inlineStr">
         <is>
           <t>Yreald Romero</t>
@@ -1114,8 +1128,9 @@
       <c r="G15" t="n">
         <v>0</v>
       </c>
-    </row>
-    <row r="16">
+      <c r="I15" s="19" t="n"/>
+    </row>
+    <row r="16" ht="18" customHeight="1" s="12">
       <c r="A16" t="inlineStr">
         <is>
           <t>Yreald Romero</t>
@@ -1141,8 +1156,9 @@
       <c r="G16" t="n">
         <v>0</v>
       </c>
-    </row>
-    <row r="17">
+      <c r="I16" s="19" t="n"/>
+    </row>
+    <row r="17" ht="18" customHeight="1" s="12">
       <c r="A17" t="inlineStr">
         <is>
           <t>Yreald Romero</t>
@@ -1168,8 +1184,9 @@
       <c r="G17" t="n">
         <v>0</v>
       </c>
-    </row>
-    <row r="18">
+      <c r="I17" s="19" t="n"/>
+    </row>
+    <row r="18" ht="18" customHeight="1" s="12">
       <c r="A18" t="inlineStr">
         <is>
           <t>Yreald Romero</t>
@@ -1195,8 +1212,9 @@
       <c r="G18" t="n">
         <v>0</v>
       </c>
-    </row>
-    <row r="19">
+      <c r="I18" s="19" t="n"/>
+    </row>
+    <row r="19" ht="18" customHeight="1" s="12">
       <c r="A19" t="inlineStr">
         <is>
           <t>Yreald Romero</t>
@@ -1222,8 +1240,9 @@
       <c r="G19" t="n">
         <v>0</v>
       </c>
-    </row>
-    <row r="20">
+      <c r="I19" s="19" t="n"/>
+    </row>
+    <row r="20" ht="18" customHeight="1" s="12">
       <c r="A20" t="inlineStr">
         <is>
           <t>Yreald Romero</t>
@@ -1249,8 +1268,9 @@
       <c r="G20" t="n">
         <v>0</v>
       </c>
-    </row>
-    <row r="21">
+      <c r="I20" s="19" t="n"/>
+    </row>
+    <row r="21" ht="18" customHeight="1" s="12">
       <c r="A21" t="inlineStr">
         <is>
           <t>Yreald Romero</t>
@@ -1276,8 +1296,9 @@
       <c r="G21" t="n">
         <v>0</v>
       </c>
-    </row>
-    <row r="22">
+      <c r="I21" s="19" t="n"/>
+    </row>
+    <row r="22" ht="18" customHeight="1" s="12">
       <c r="A22" t="inlineStr">
         <is>
           <t>Yreald Romero</t>
@@ -1303,8 +1324,9 @@
       <c r="G22" t="n">
         <v>0</v>
       </c>
-    </row>
-    <row r="23">
+      <c r="I22" s="19" t="n"/>
+    </row>
+    <row r="23" ht="18" customHeight="1" s="12">
       <c r="A23" t="inlineStr">
         <is>
           <t>Yreald Romero</t>
@@ -1330,8 +1352,9 @@
       <c r="G23" t="n">
         <v>0</v>
       </c>
-    </row>
-    <row r="24">
+      <c r="I23" s="19" t="n"/>
+    </row>
+    <row r="24" ht="18" customHeight="1" s="12">
       <c r="A24" t="inlineStr">
         <is>
           <t>Yreald Romero</t>
@@ -1357,8 +1380,9 @@
       <c r="G24" t="n">
         <v>0</v>
       </c>
-    </row>
-    <row r="25">
+      <c r="I24" s="19" t="n"/>
+    </row>
+    <row r="25" ht="18" customHeight="1" s="12">
       <c r="A25" t="inlineStr">
         <is>
           <t>Yreald Romero</t>
@@ -1384,6 +1408,1432 @@
       <c r="G25" t="n">
         <v>0</v>
       </c>
+      <c r="I25" s="19" t="n"/>
+    </row>
+    <row r="26" ht="18" customHeight="1" s="12">
+      <c r="I26" s="19" t="n"/>
+    </row>
+    <row r="27" ht="18" customHeight="1" s="12">
+      <c r="I27" s="19" t="n"/>
+    </row>
+    <row r="28" ht="18" customHeight="1" s="12">
+      <c r="I28" s="19" t="n"/>
+    </row>
+    <row r="29" ht="18" customHeight="1" s="12">
+      <c r="I29" s="19" t="n"/>
+    </row>
+    <row r="30" ht="18" customHeight="1" s="12">
+      <c r="I30" s="19" t="n"/>
+    </row>
+    <row r="31" ht="18" customHeight="1" s="12">
+      <c r="I31" s="19" t="n"/>
+    </row>
+    <row r="32" ht="18" customHeight="1" s="12">
+      <c r="I32" s="19" t="n"/>
+    </row>
+    <row r="33" ht="18" customHeight="1" s="12">
+      <c r="I33" s="19" t="n"/>
+    </row>
+    <row r="34" ht="18" customHeight="1" s="12">
+      <c r="I34" s="19" t="n"/>
+    </row>
+    <row r="35" ht="18" customHeight="1" s="12">
+      <c r="I35" s="19" t="n"/>
+    </row>
+    <row r="36" ht="18" customHeight="1" s="12">
+      <c r="I36" s="19" t="n"/>
+    </row>
+    <row r="37" ht="18" customHeight="1" s="12">
+      <c r="I37" s="19" t="n"/>
+    </row>
+    <row r="38" ht="18" customHeight="1" s="12">
+      <c r="I38" s="19" t="n"/>
+    </row>
+    <row r="39" ht="18" customHeight="1" s="12">
+      <c r="I39" s="19" t="n"/>
+    </row>
+    <row r="40" ht="18" customHeight="1" s="12">
+      <c r="I40" s="19" t="n"/>
+    </row>
+    <row r="41" ht="18" customHeight="1" s="12">
+      <c r="I41" s="19" t="n"/>
+    </row>
+    <row r="42" ht="18" customHeight="1" s="12">
+      <c r="I42" s="19" t="n"/>
+    </row>
+    <row r="43" ht="18" customHeight="1" s="12">
+      <c r="I43" s="19" t="n"/>
+    </row>
+    <row r="44" ht="18" customHeight="1" s="12">
+      <c r="I44" s="19" t="n"/>
+    </row>
+    <row r="45" ht="18" customHeight="1" s="12">
+      <c r="I45" s="19" t="n"/>
+    </row>
+    <row r="46" ht="18" customHeight="1" s="12">
+      <c r="I46" s="19" t="n"/>
+    </row>
+    <row r="47" ht="18" customHeight="1" s="12">
+      <c r="I47" s="19" t="n"/>
+    </row>
+    <row r="48" ht="18" customHeight="1" s="12">
+      <c r="I48" s="19" t="n"/>
+    </row>
+    <row r="49" ht="18" customHeight="1" s="12">
+      <c r="I49" s="19" t="n"/>
+    </row>
+    <row r="50" ht="18" customHeight="1" s="12">
+      <c r="I50" s="19" t="n"/>
+    </row>
+    <row r="51" ht="18" customHeight="1" s="12">
+      <c r="I51" s="19" t="n"/>
+    </row>
+    <row r="52" ht="18" customHeight="1" s="12">
+      <c r="I52" s="19" t="n"/>
+    </row>
+    <row r="53" ht="18" customHeight="1" s="12">
+      <c r="I53" s="19" t="n"/>
+    </row>
+    <row r="54" ht="18" customHeight="1" s="12">
+      <c r="I54" s="19" t="n"/>
+    </row>
+    <row r="55" ht="18" customHeight="1" s="12">
+      <c r="I55" s="19" t="n"/>
+    </row>
+    <row r="56" ht="18" customHeight="1" s="12">
+      <c r="I56" s="19" t="n"/>
+    </row>
+    <row r="57" ht="18" customHeight="1" s="12">
+      <c r="I57" s="19" t="n"/>
+    </row>
+    <row r="58" ht="18" customHeight="1" s="12">
+      <c r="I58" s="19" t="n"/>
+    </row>
+    <row r="59" ht="18" customHeight="1" s="12">
+      <c r="I59" s="19" t="n"/>
+    </row>
+    <row r="60" ht="18" customHeight="1" s="12">
+      <c r="I60" s="19" t="n"/>
+    </row>
+    <row r="61" ht="18" customHeight="1" s="12">
+      <c r="I61" s="19" t="n"/>
+    </row>
+    <row r="62" ht="18" customHeight="1" s="12">
+      <c r="I62" s="19" t="n"/>
+    </row>
+    <row r="63" ht="18" customHeight="1" s="12">
+      <c r="I63" s="19" t="n"/>
+    </row>
+    <row r="64" ht="18" customHeight="1" s="12">
+      <c r="I64" s="19" t="n"/>
+    </row>
+    <row r="65" ht="18" customHeight="1" s="12">
+      <c r="I65" s="19" t="n"/>
+    </row>
+    <row r="66" ht="18" customHeight="1" s="12">
+      <c r="I66" s="19" t="n"/>
+    </row>
+    <row r="67" ht="18" customHeight="1" s="12">
+      <c r="I67" s="19" t="n"/>
+    </row>
+    <row r="68" ht="18" customHeight="1" s="12">
+      <c r="I68" s="19" t="n"/>
+    </row>
+    <row r="69" ht="18" customHeight="1" s="12">
+      <c r="I69" s="19" t="n"/>
+    </row>
+    <row r="70" ht="18" customHeight="1" s="12">
+      <c r="I70" s="19" t="n"/>
+    </row>
+    <row r="71" ht="18" customHeight="1" s="12">
+      <c r="I71" s="19" t="n"/>
+    </row>
+    <row r="72" ht="18" customHeight="1" s="12">
+      <c r="I72" s="19" t="n"/>
+    </row>
+    <row r="73" ht="18" customHeight="1" s="12">
+      <c r="I73" s="19" t="n"/>
+    </row>
+    <row r="74" ht="18" customHeight="1" s="12">
+      <c r="I74" s="19" t="n"/>
+    </row>
+    <row r="75" ht="18" customHeight="1" s="12">
+      <c r="I75" s="19" t="n"/>
+    </row>
+    <row r="76" ht="18" customHeight="1" s="12">
+      <c r="I76" s="19" t="n"/>
+    </row>
+    <row r="77" ht="18" customHeight="1" s="12">
+      <c r="I77" s="19" t="n"/>
+    </row>
+    <row r="78" ht="18" customHeight="1" s="12">
+      <c r="I78" s="19" t="n"/>
+    </row>
+    <row r="79" ht="18" customHeight="1" s="12">
+      <c r="I79" s="19" t="n"/>
+    </row>
+    <row r="80" ht="18" customHeight="1" s="12">
+      <c r="I80" s="19" t="n"/>
+    </row>
+    <row r="81" ht="18" customHeight="1" s="12">
+      <c r="I81" s="19" t="n"/>
+    </row>
+    <row r="82" ht="18" customHeight="1" s="12">
+      <c r="I82" s="19" t="n"/>
+    </row>
+    <row r="83" ht="18" customHeight="1" s="12">
+      <c r="I83" s="19" t="n"/>
+    </row>
+    <row r="84" ht="18" customHeight="1" s="12">
+      <c r="I84" s="19" t="n"/>
+    </row>
+    <row r="85" ht="18" customHeight="1" s="12">
+      <c r="I85" s="19" t="n"/>
+    </row>
+    <row r="86" ht="18" customHeight="1" s="12">
+      <c r="I86" s="19" t="n"/>
+    </row>
+    <row r="87" ht="18" customHeight="1" s="12">
+      <c r="I87" s="19" t="n"/>
+    </row>
+    <row r="88" ht="18" customHeight="1" s="12">
+      <c r="I88" s="19" t="n"/>
+    </row>
+    <row r="89" ht="18" customHeight="1" s="12">
+      <c r="I89" s="19" t="n"/>
+    </row>
+    <row r="90" ht="18" customHeight="1" s="12">
+      <c r="I90" s="19" t="n"/>
+    </row>
+    <row r="91" ht="18" customHeight="1" s="12">
+      <c r="I91" s="19" t="n"/>
+    </row>
+    <row r="92" ht="18" customHeight="1" s="12">
+      <c r="I92" s="19" t="n"/>
+    </row>
+    <row r="93" ht="18" customHeight="1" s="12">
+      <c r="I93" s="19" t="n"/>
+    </row>
+    <row r="94" ht="18" customHeight="1" s="12">
+      <c r="I94" s="19" t="n"/>
+    </row>
+    <row r="95" ht="18" customHeight="1" s="12">
+      <c r="I95" s="19" t="n"/>
+    </row>
+    <row r="96" ht="18" customHeight="1" s="12">
+      <c r="I96" s="19" t="n"/>
+    </row>
+    <row r="97" ht="18" customHeight="1" s="12">
+      <c r="I97" s="19" t="n"/>
+    </row>
+    <row r="98" ht="18" customHeight="1" s="12">
+      <c r="I98" s="19" t="n"/>
+    </row>
+    <row r="99" ht="18" customHeight="1" s="12">
+      <c r="I99" s="19" t="n"/>
+    </row>
+    <row r="100" ht="18" customHeight="1" s="12">
+      <c r="I100" s="19" t="n"/>
+    </row>
+    <row r="101" ht="18" customHeight="1" s="12">
+      <c r="I101" s="19" t="n"/>
+    </row>
+    <row r="102" ht="18" customHeight="1" s="12">
+      <c r="I102" s="19" t="n"/>
+    </row>
+    <row r="103" ht="18" customHeight="1" s="12">
+      <c r="I103" s="19" t="n"/>
+    </row>
+    <row r="104" ht="18" customHeight="1" s="12">
+      <c r="I104" s="19" t="n"/>
+    </row>
+    <row r="105" ht="18" customHeight="1" s="12">
+      <c r="I105" s="19" t="n"/>
+    </row>
+    <row r="106" ht="18" customHeight="1" s="12">
+      <c r="I106" s="19" t="n"/>
+    </row>
+    <row r="107" ht="18" customHeight="1" s="12">
+      <c r="I107" s="19" t="n"/>
+    </row>
+    <row r="108" ht="18" customHeight="1" s="12">
+      <c r="I108" s="19" t="n"/>
+    </row>
+    <row r="109" ht="18" customHeight="1" s="12">
+      <c r="I109" s="19" t="n"/>
+    </row>
+    <row r="110" ht="18" customHeight="1" s="12">
+      <c r="I110" s="19" t="n"/>
+    </row>
+    <row r="111" ht="18" customHeight="1" s="12">
+      <c r="I111" s="19" t="n"/>
+    </row>
+    <row r="112" ht="18" customHeight="1" s="12">
+      <c r="I112" s="19" t="n"/>
+    </row>
+    <row r="113" ht="18" customHeight="1" s="12">
+      <c r="I113" s="19" t="n"/>
+    </row>
+    <row r="114" ht="18" customHeight="1" s="12">
+      <c r="I114" s="19" t="n"/>
+    </row>
+    <row r="115" ht="18" customHeight="1" s="12">
+      <c r="I115" s="19" t="n"/>
+    </row>
+    <row r="116" ht="18" customHeight="1" s="12">
+      <c r="I116" s="19" t="n"/>
+    </row>
+    <row r="117" ht="18" customHeight="1" s="12">
+      <c r="I117" s="19" t="n"/>
+    </row>
+    <row r="118" ht="18" customHeight="1" s="12">
+      <c r="I118" s="19" t="n"/>
+    </row>
+    <row r="119" ht="18" customHeight="1" s="12">
+      <c r="I119" s="19" t="n"/>
+    </row>
+    <row r="120" ht="18" customHeight="1" s="12">
+      <c r="I120" s="19" t="n"/>
+    </row>
+    <row r="121" ht="18" customHeight="1" s="12">
+      <c r="I121" s="19" t="n"/>
+    </row>
+    <row r="122" ht="18" customHeight="1" s="12">
+      <c r="I122" s="19" t="n"/>
+    </row>
+    <row r="123" ht="18" customHeight="1" s="12">
+      <c r="I123" s="19" t="n"/>
+    </row>
+    <row r="124" ht="18" customHeight="1" s="12">
+      <c r="I124" s="19" t="n"/>
+    </row>
+    <row r="125" ht="18" customHeight="1" s="12">
+      <c r="I125" s="19" t="n"/>
+    </row>
+    <row r="126" ht="18" customHeight="1" s="12">
+      <c r="I126" s="19" t="n"/>
+    </row>
+    <row r="127" ht="18" customHeight="1" s="12">
+      <c r="I127" s="19" t="n"/>
+    </row>
+    <row r="128" ht="18" customHeight="1" s="12">
+      <c r="I128" s="19" t="n"/>
+    </row>
+    <row r="129" ht="18" customHeight="1" s="12">
+      <c r="I129" s="19" t="n"/>
+    </row>
+    <row r="130" ht="18" customHeight="1" s="12">
+      <c r="I130" s="19" t="n"/>
+    </row>
+    <row r="131" ht="18" customHeight="1" s="12">
+      <c r="I131" s="19" t="n"/>
+    </row>
+    <row r="132" ht="18" customHeight="1" s="12">
+      <c r="I132" s="19" t="n"/>
+    </row>
+    <row r="133" ht="18" customHeight="1" s="12">
+      <c r="I133" s="19" t="n"/>
+    </row>
+    <row r="134" ht="18" customHeight="1" s="12">
+      <c r="I134" s="19" t="n"/>
+    </row>
+    <row r="135" ht="18" customHeight="1" s="12">
+      <c r="I135" s="19" t="n"/>
+    </row>
+    <row r="136" ht="18" customHeight="1" s="12">
+      <c r="I136" s="19" t="n"/>
+    </row>
+    <row r="137" ht="18" customHeight="1" s="12">
+      <c r="I137" s="19" t="n"/>
+    </row>
+    <row r="138" ht="18" customHeight="1" s="12">
+      <c r="I138" s="19" t="n"/>
+    </row>
+    <row r="139" ht="18" customHeight="1" s="12">
+      <c r="I139" s="19" t="n"/>
+    </row>
+    <row r="140" ht="18" customHeight="1" s="12">
+      <c r="I140" s="19" t="n"/>
+    </row>
+    <row r="141" ht="18" customHeight="1" s="12">
+      <c r="I141" s="19" t="n"/>
+    </row>
+    <row r="142" ht="18" customHeight="1" s="12">
+      <c r="I142" s="19" t="n"/>
+    </row>
+    <row r="143" ht="18" customHeight="1" s="12">
+      <c r="I143" s="19" t="n"/>
+    </row>
+    <row r="144" ht="18" customHeight="1" s="12">
+      <c r="I144" s="19" t="n"/>
+    </row>
+    <row r="145" ht="18" customHeight="1" s="12">
+      <c r="I145" s="19" t="n"/>
+    </row>
+    <row r="146" ht="18" customHeight="1" s="12">
+      <c r="I146" s="19" t="n"/>
+    </row>
+    <row r="147" ht="18" customHeight="1" s="12">
+      <c r="I147" s="19" t="n"/>
+    </row>
+    <row r="148" ht="18" customHeight="1" s="12">
+      <c r="I148" s="19" t="n"/>
+    </row>
+    <row r="149" ht="18" customHeight="1" s="12">
+      <c r="I149" s="19" t="n"/>
+    </row>
+    <row r="150" ht="18" customHeight="1" s="12">
+      <c r="I150" s="19" t="n"/>
+    </row>
+    <row r="151" ht="18" customHeight="1" s="12">
+      <c r="I151" s="19" t="n"/>
+    </row>
+    <row r="152" ht="18" customHeight="1" s="12">
+      <c r="I152" s="19" t="n"/>
+    </row>
+    <row r="153" ht="18" customHeight="1" s="12">
+      <c r="I153" s="19" t="n"/>
+    </row>
+    <row r="154" ht="18" customHeight="1" s="12">
+      <c r="I154" s="19" t="n"/>
+    </row>
+    <row r="155" ht="18" customHeight="1" s="12">
+      <c r="I155" s="19" t="n"/>
+    </row>
+    <row r="156" ht="18" customHeight="1" s="12">
+      <c r="I156" s="19" t="n"/>
+    </row>
+    <row r="157" ht="18" customHeight="1" s="12">
+      <c r="I157" s="19" t="n"/>
+    </row>
+    <row r="158" ht="18" customHeight="1" s="12">
+      <c r="I158" s="19" t="n"/>
+    </row>
+    <row r="159" ht="18" customHeight="1" s="12">
+      <c r="I159" s="19" t="n"/>
+    </row>
+    <row r="160" ht="18" customHeight="1" s="12">
+      <c r="I160" s="19" t="n"/>
+    </row>
+    <row r="161" ht="18" customHeight="1" s="12">
+      <c r="I161" s="19" t="n"/>
+    </row>
+    <row r="162" ht="18" customHeight="1" s="12">
+      <c r="I162" s="19" t="n"/>
+    </row>
+    <row r="163" ht="18" customHeight="1" s="12">
+      <c r="I163" s="19" t="n"/>
+    </row>
+    <row r="164" ht="18" customHeight="1" s="12">
+      <c r="I164" s="19" t="n"/>
+    </row>
+    <row r="165" ht="18" customHeight="1" s="12">
+      <c r="I165" s="19" t="n"/>
+    </row>
+    <row r="166" ht="18" customHeight="1" s="12">
+      <c r="I166" s="19" t="n"/>
+    </row>
+    <row r="167" ht="18" customHeight="1" s="12">
+      <c r="I167" s="19" t="n"/>
+    </row>
+    <row r="168" ht="18" customHeight="1" s="12">
+      <c r="I168" s="19" t="n"/>
+    </row>
+    <row r="169" ht="18" customHeight="1" s="12">
+      <c r="I169" s="19" t="n"/>
+    </row>
+    <row r="170" ht="18" customHeight="1" s="12">
+      <c r="I170" s="19" t="n"/>
+    </row>
+    <row r="171" ht="18" customHeight="1" s="12">
+      <c r="I171" s="19" t="n"/>
+    </row>
+    <row r="172" ht="18" customHeight="1" s="12">
+      <c r="I172" s="19" t="n"/>
+    </row>
+    <row r="173" ht="18" customHeight="1" s="12">
+      <c r="I173" s="19" t="n"/>
+    </row>
+    <row r="174" ht="18" customHeight="1" s="12">
+      <c r="I174" s="19" t="n"/>
+    </row>
+    <row r="175" ht="18" customHeight="1" s="12">
+      <c r="I175" s="19" t="n"/>
+    </row>
+    <row r="176" ht="18" customHeight="1" s="12">
+      <c r="I176" s="19" t="n"/>
+    </row>
+    <row r="177" ht="18" customHeight="1" s="12">
+      <c r="I177" s="19" t="n"/>
+    </row>
+    <row r="178" ht="18" customHeight="1" s="12">
+      <c r="I178" s="19" t="n"/>
+    </row>
+    <row r="179" ht="18" customHeight="1" s="12">
+      <c r="I179" s="19" t="n"/>
+    </row>
+    <row r="180" ht="18" customHeight="1" s="12">
+      <c r="I180" s="19" t="n"/>
+    </row>
+    <row r="181" ht="18" customHeight="1" s="12">
+      <c r="I181" s="19" t="n"/>
+    </row>
+    <row r="182" ht="18" customHeight="1" s="12">
+      <c r="I182" s="19" t="n"/>
+    </row>
+    <row r="183" ht="18" customHeight="1" s="12">
+      <c r="I183" s="19" t="n"/>
+    </row>
+    <row r="184" ht="18" customHeight="1" s="12">
+      <c r="I184" s="19" t="n"/>
+    </row>
+    <row r="185" ht="18" customHeight="1" s="12">
+      <c r="I185" s="19" t="n"/>
+    </row>
+    <row r="186" ht="18" customHeight="1" s="12">
+      <c r="I186" s="19" t="n"/>
+    </row>
+    <row r="187" ht="18" customHeight="1" s="12">
+      <c r="I187" s="19" t="n"/>
+    </row>
+    <row r="188" ht="18" customHeight="1" s="12">
+      <c r="I188" s="19" t="n"/>
+    </row>
+    <row r="189" ht="18" customHeight="1" s="12">
+      <c r="I189" s="19" t="n"/>
+    </row>
+    <row r="190" ht="18" customHeight="1" s="12">
+      <c r="I190" s="19" t="n"/>
+    </row>
+    <row r="191" ht="18" customHeight="1" s="12">
+      <c r="I191" s="19" t="n"/>
+    </row>
+    <row r="192" ht="18" customHeight="1" s="12">
+      <c r="I192" s="19" t="n"/>
+    </row>
+    <row r="193" ht="18" customHeight="1" s="12">
+      <c r="I193" s="19" t="n"/>
+    </row>
+    <row r="194" ht="18" customHeight="1" s="12">
+      <c r="I194" s="19" t="n"/>
+    </row>
+    <row r="195" ht="18" customHeight="1" s="12">
+      <c r="I195" s="19" t="n"/>
+    </row>
+    <row r="196" ht="18" customHeight="1" s="12">
+      <c r="I196" s="19" t="n"/>
+    </row>
+    <row r="197" ht="18" customHeight="1" s="12">
+      <c r="I197" s="19" t="n"/>
+    </row>
+    <row r="198" ht="18" customHeight="1" s="12">
+      <c r="I198" s="19" t="n"/>
+    </row>
+    <row r="199" ht="18" customHeight="1" s="12">
+      <c r="I199" s="19" t="n"/>
+    </row>
+    <row r="200" ht="18" customHeight="1" s="12">
+      <c r="I200" s="19" t="n"/>
+    </row>
+    <row r="201" ht="18" customHeight="1" s="12">
+      <c r="I201" s="19" t="n"/>
+    </row>
+    <row r="202" ht="18" customHeight="1" s="12">
+      <c r="I202" s="19" t="n"/>
+    </row>
+    <row r="203" ht="18" customHeight="1" s="12">
+      <c r="I203" s="19" t="n"/>
+    </row>
+    <row r="204" ht="18" customHeight="1" s="12">
+      <c r="I204" s="19" t="n"/>
+    </row>
+    <row r="205" ht="18" customHeight="1" s="12">
+      <c r="I205" s="19" t="n"/>
+    </row>
+    <row r="206" ht="18" customHeight="1" s="12">
+      <c r="I206" s="19" t="n"/>
+    </row>
+    <row r="207" ht="18" customHeight="1" s="12">
+      <c r="I207" s="19" t="n"/>
+    </row>
+    <row r="208" ht="18" customHeight="1" s="12">
+      <c r="I208" s="19" t="n"/>
+    </row>
+    <row r="209" ht="18" customHeight="1" s="12">
+      <c r="I209" s="19" t="n"/>
+    </row>
+    <row r="210" ht="18" customHeight="1" s="12">
+      <c r="I210" s="19" t="n"/>
+    </row>
+    <row r="211" ht="18" customHeight="1" s="12">
+      <c r="I211" s="19" t="n"/>
+    </row>
+    <row r="212" ht="18" customHeight="1" s="12">
+      <c r="I212" s="19" t="n"/>
+    </row>
+    <row r="213" ht="18" customHeight="1" s="12">
+      <c r="I213" s="19" t="n"/>
+    </row>
+    <row r="214" ht="18" customHeight="1" s="12">
+      <c r="I214" s="19" t="n"/>
+    </row>
+    <row r="215" ht="18" customHeight="1" s="12">
+      <c r="I215" s="19" t="n"/>
+    </row>
+    <row r="216" ht="18" customHeight="1" s="12">
+      <c r="I216" s="19" t="n"/>
+    </row>
+    <row r="217" ht="18" customHeight="1" s="12">
+      <c r="I217" s="19" t="n"/>
+    </row>
+    <row r="218" ht="18" customHeight="1" s="12">
+      <c r="I218" s="19" t="n"/>
+    </row>
+    <row r="219" ht="18" customHeight="1" s="12">
+      <c r="I219" s="19" t="n"/>
+    </row>
+    <row r="220" ht="18" customHeight="1" s="12">
+      <c r="I220" s="19" t="n"/>
+    </row>
+    <row r="221" ht="18" customHeight="1" s="12">
+      <c r="I221" s="19" t="n"/>
+    </row>
+    <row r="222" ht="18" customHeight="1" s="12">
+      <c r="I222" s="19" t="n"/>
+    </row>
+    <row r="223" ht="18" customHeight="1" s="12">
+      <c r="I223" s="19" t="n"/>
+    </row>
+    <row r="224" ht="18" customHeight="1" s="12">
+      <c r="I224" s="19" t="n"/>
+    </row>
+    <row r="225" ht="18" customHeight="1" s="12">
+      <c r="I225" s="19" t="n"/>
+    </row>
+    <row r="226" ht="18" customHeight="1" s="12">
+      <c r="I226" s="19" t="n"/>
+    </row>
+    <row r="227" ht="18" customHeight="1" s="12">
+      <c r="I227" s="19" t="n"/>
+    </row>
+    <row r="228" ht="18" customHeight="1" s="12">
+      <c r="I228" s="19" t="n"/>
+    </row>
+    <row r="229" ht="18" customHeight="1" s="12">
+      <c r="I229" s="19" t="n"/>
+    </row>
+    <row r="230" ht="18" customHeight="1" s="12">
+      <c r="I230" s="19" t="n"/>
+    </row>
+    <row r="231" ht="18" customHeight="1" s="12">
+      <c r="I231" s="19" t="n"/>
+    </row>
+    <row r="232" ht="18" customHeight="1" s="12">
+      <c r="I232" s="19" t="n"/>
+    </row>
+    <row r="233" ht="18" customHeight="1" s="12">
+      <c r="I233" s="19" t="n"/>
+    </row>
+    <row r="234" ht="18" customHeight="1" s="12">
+      <c r="I234" s="19" t="n"/>
+    </row>
+    <row r="235" ht="18" customHeight="1" s="12">
+      <c r="I235" s="19" t="n"/>
+    </row>
+    <row r="236" ht="18" customHeight="1" s="12">
+      <c r="I236" s="19" t="n"/>
+    </row>
+    <row r="237" ht="18" customHeight="1" s="12">
+      <c r="I237" s="19" t="n"/>
+    </row>
+    <row r="238" ht="18" customHeight="1" s="12">
+      <c r="I238" s="19" t="n"/>
+    </row>
+    <row r="239" ht="18" customHeight="1" s="12">
+      <c r="I239" s="19" t="n"/>
+    </row>
+    <row r="240" ht="18" customHeight="1" s="12">
+      <c r="I240" s="19" t="n"/>
+    </row>
+    <row r="241" ht="18" customHeight="1" s="12">
+      <c r="I241" s="19" t="n"/>
+    </row>
+    <row r="242" ht="18" customHeight="1" s="12">
+      <c r="I242" s="19" t="n"/>
+    </row>
+    <row r="243" ht="18" customHeight="1" s="12">
+      <c r="I243" s="19" t="n"/>
+    </row>
+    <row r="244" ht="18" customHeight="1" s="12">
+      <c r="I244" s="19" t="n"/>
+    </row>
+    <row r="245" ht="18" customHeight="1" s="12">
+      <c r="I245" s="19" t="n"/>
+    </row>
+    <row r="246" ht="18" customHeight="1" s="12">
+      <c r="I246" s="19" t="n"/>
+    </row>
+    <row r="247" ht="18" customHeight="1" s="12">
+      <c r="I247" s="19" t="n"/>
+    </row>
+    <row r="248" ht="18" customHeight="1" s="12">
+      <c r="I248" s="19" t="n"/>
+    </row>
+    <row r="249" ht="18" customHeight="1" s="12">
+      <c r="I249" s="19" t="n"/>
+    </row>
+    <row r="250" ht="18" customHeight="1" s="12">
+      <c r="I250" s="19" t="n"/>
+    </row>
+    <row r="251" ht="18" customHeight="1" s="12">
+      <c r="I251" s="19" t="n"/>
+    </row>
+    <row r="252" ht="18" customHeight="1" s="12">
+      <c r="I252" s="19" t="n"/>
+    </row>
+    <row r="253" ht="18" customHeight="1" s="12">
+      <c r="I253" s="19" t="n"/>
+    </row>
+    <row r="254" ht="18" customHeight="1" s="12">
+      <c r="I254" s="19" t="n"/>
+    </row>
+    <row r="255" ht="18" customHeight="1" s="12">
+      <c r="I255" s="19" t="n"/>
+    </row>
+    <row r="256" ht="18" customHeight="1" s="12">
+      <c r="I256" s="19" t="n"/>
+    </row>
+    <row r="257" ht="18" customHeight="1" s="12">
+      <c r="I257" s="19" t="n"/>
+    </row>
+    <row r="258" ht="18" customHeight="1" s="12">
+      <c r="I258" s="19" t="n"/>
+    </row>
+    <row r="259" ht="18" customHeight="1" s="12">
+      <c r="I259" s="19" t="n"/>
+    </row>
+    <row r="260" ht="18" customHeight="1" s="12">
+      <c r="I260" s="19" t="n"/>
+    </row>
+    <row r="261" ht="18" customHeight="1" s="12">
+      <c r="I261" s="19" t="n"/>
+    </row>
+    <row r="262" ht="18" customHeight="1" s="12">
+      <c r="I262" s="19" t="n"/>
+    </row>
+    <row r="263" ht="18" customHeight="1" s="12">
+      <c r="I263" s="19" t="n"/>
+    </row>
+    <row r="264" ht="18" customHeight="1" s="12">
+      <c r="I264" s="19" t="n"/>
+    </row>
+    <row r="265" ht="18" customHeight="1" s="12">
+      <c r="I265" s="19" t="n"/>
+    </row>
+    <row r="266" ht="18" customHeight="1" s="12">
+      <c r="I266" s="19" t="n"/>
+    </row>
+    <row r="267" ht="18" customHeight="1" s="12">
+      <c r="I267" s="19" t="n"/>
+    </row>
+    <row r="268" ht="18" customHeight="1" s="12">
+      <c r="I268" s="19" t="n"/>
+    </row>
+    <row r="269" ht="18" customHeight="1" s="12">
+      <c r="I269" s="19" t="n"/>
+    </row>
+    <row r="270" ht="18" customHeight="1" s="12">
+      <c r="I270" s="19" t="n"/>
+    </row>
+    <row r="271" ht="18" customHeight="1" s="12">
+      <c r="I271" s="19" t="n"/>
+    </row>
+    <row r="272" ht="18" customHeight="1" s="12">
+      <c r="I272" s="19" t="n"/>
+    </row>
+    <row r="273" ht="18" customHeight="1" s="12">
+      <c r="I273" s="19" t="n"/>
+    </row>
+    <row r="274" ht="18" customHeight="1" s="12">
+      <c r="I274" s="19" t="n"/>
+    </row>
+    <row r="275" ht="18" customHeight="1" s="12">
+      <c r="I275" s="19" t="n"/>
+    </row>
+    <row r="276" ht="18" customHeight="1" s="12">
+      <c r="I276" s="19" t="n"/>
+    </row>
+    <row r="277" ht="18" customHeight="1" s="12">
+      <c r="I277" s="19" t="n"/>
+    </row>
+    <row r="278" ht="18" customHeight="1" s="12">
+      <c r="I278" s="19" t="n"/>
+    </row>
+    <row r="279" ht="18" customHeight="1" s="12">
+      <c r="I279" s="19" t="n"/>
+    </row>
+    <row r="280" ht="18" customHeight="1" s="12">
+      <c r="I280" s="19" t="n"/>
+    </row>
+    <row r="281" ht="18" customHeight="1" s="12">
+      <c r="I281" s="19" t="n"/>
+    </row>
+    <row r="282" ht="18" customHeight="1" s="12">
+      <c r="I282" s="19" t="n"/>
+    </row>
+    <row r="283" ht="18" customHeight="1" s="12">
+      <c r="I283" s="19" t="n"/>
+    </row>
+    <row r="284" ht="18" customHeight="1" s="12">
+      <c r="I284" s="19" t="n"/>
+    </row>
+    <row r="285" ht="18" customHeight="1" s="12">
+      <c r="I285" s="19" t="n"/>
+    </row>
+    <row r="286" ht="18" customHeight="1" s="12">
+      <c r="I286" s="19" t="n"/>
+    </row>
+    <row r="287" ht="18" customHeight="1" s="12">
+      <c r="I287" s="19" t="n"/>
+    </row>
+    <row r="288" ht="18" customHeight="1" s="12">
+      <c r="I288" s="19" t="n"/>
+    </row>
+    <row r="289" ht="18" customHeight="1" s="12">
+      <c r="I289" s="19" t="n"/>
+    </row>
+    <row r="290" ht="18" customHeight="1" s="12">
+      <c r="I290" s="19" t="n"/>
+    </row>
+    <row r="291" ht="18" customHeight="1" s="12">
+      <c r="I291" s="19" t="n"/>
+    </row>
+    <row r="292" ht="18" customHeight="1" s="12">
+      <c r="I292" s="19" t="n"/>
+    </row>
+    <row r="293" ht="18" customHeight="1" s="12">
+      <c r="I293" s="19" t="n"/>
+    </row>
+    <row r="294" ht="18" customHeight="1" s="12">
+      <c r="I294" s="19" t="n"/>
+    </row>
+    <row r="295" ht="18" customHeight="1" s="12">
+      <c r="I295" s="19" t="n"/>
+    </row>
+    <row r="296" ht="18" customHeight="1" s="12">
+      <c r="I296" s="19" t="n"/>
+    </row>
+    <row r="297" ht="18" customHeight="1" s="12">
+      <c r="I297" s="19" t="n"/>
+    </row>
+    <row r="298" ht="18" customHeight="1" s="12">
+      <c r="I298" s="19" t="n"/>
+    </row>
+    <row r="299" ht="18" customHeight="1" s="12">
+      <c r="I299" s="19" t="n"/>
+    </row>
+    <row r="300" ht="18" customHeight="1" s="12">
+      <c r="I300" s="19" t="n"/>
+    </row>
+    <row r="301" ht="18" customHeight="1" s="12">
+      <c r="I301" s="19" t="n"/>
+    </row>
+    <row r="302" ht="18" customHeight="1" s="12">
+      <c r="I302" s="19" t="n"/>
+    </row>
+    <row r="303" ht="18" customHeight="1" s="12">
+      <c r="I303" s="19" t="n"/>
+    </row>
+    <row r="304" ht="18" customHeight="1" s="12">
+      <c r="I304" s="19" t="n"/>
+    </row>
+    <row r="305" ht="18" customHeight="1" s="12">
+      <c r="I305" s="19" t="n"/>
+    </row>
+    <row r="306" ht="18" customHeight="1" s="12">
+      <c r="I306" s="19" t="n"/>
+    </row>
+    <row r="307" ht="18" customHeight="1" s="12">
+      <c r="I307" s="19" t="n"/>
+    </row>
+    <row r="308" ht="18" customHeight="1" s="12">
+      <c r="I308" s="19" t="n"/>
+    </row>
+    <row r="309" ht="18" customHeight="1" s="12">
+      <c r="I309" s="19" t="n"/>
+    </row>
+    <row r="310" ht="18" customHeight="1" s="12">
+      <c r="I310" s="19" t="n"/>
+    </row>
+    <row r="311" ht="18" customHeight="1" s="12">
+      <c r="I311" s="19" t="n"/>
+    </row>
+    <row r="312" ht="18" customHeight="1" s="12">
+      <c r="I312" s="19" t="n"/>
+    </row>
+    <row r="313" ht="18" customHeight="1" s="12">
+      <c r="I313" s="19" t="n"/>
+    </row>
+    <row r="314" ht="18" customHeight="1" s="12">
+      <c r="I314" s="19" t="n"/>
+    </row>
+    <row r="315" ht="18" customHeight="1" s="12">
+      <c r="I315" s="19" t="n"/>
+    </row>
+    <row r="316" ht="18" customHeight="1" s="12">
+      <c r="I316" s="19" t="n"/>
+    </row>
+    <row r="317" ht="18" customHeight="1" s="12">
+      <c r="I317" s="19" t="n"/>
+    </row>
+    <row r="318" ht="18" customHeight="1" s="12">
+      <c r="I318" s="19" t="n"/>
+    </row>
+    <row r="319" ht="18" customHeight="1" s="12">
+      <c r="I319" s="19" t="n"/>
+    </row>
+    <row r="320" ht="18" customHeight="1" s="12">
+      <c r="I320" s="19" t="n"/>
+    </row>
+    <row r="321" ht="18" customHeight="1" s="12">
+      <c r="I321" s="19" t="n"/>
+    </row>
+    <row r="322" ht="18" customHeight="1" s="12">
+      <c r="I322" s="19" t="n"/>
+    </row>
+    <row r="323" ht="18" customHeight="1" s="12">
+      <c r="I323" s="19" t="n"/>
+    </row>
+    <row r="324" ht="18" customHeight="1" s="12">
+      <c r="I324" s="19" t="n"/>
+    </row>
+    <row r="325" ht="18" customHeight="1" s="12">
+      <c r="I325" s="19" t="n"/>
+    </row>
+    <row r="326" ht="18" customHeight="1" s="12">
+      <c r="I326" s="19" t="n"/>
+    </row>
+    <row r="327" ht="18" customHeight="1" s="12">
+      <c r="I327" s="19" t="n"/>
+    </row>
+    <row r="328" ht="18" customHeight="1" s="12">
+      <c r="I328" s="19" t="n"/>
+    </row>
+    <row r="329" ht="18" customHeight="1" s="12">
+      <c r="I329" s="19" t="n"/>
+    </row>
+    <row r="330" ht="18" customHeight="1" s="12">
+      <c r="I330" s="19" t="n"/>
+    </row>
+    <row r="331" ht="18" customHeight="1" s="12">
+      <c r="I331" s="19" t="n"/>
+    </row>
+    <row r="332" ht="18" customHeight="1" s="12">
+      <c r="I332" s="19" t="n"/>
+    </row>
+    <row r="333" ht="18" customHeight="1" s="12">
+      <c r="I333" s="19" t="n"/>
+    </row>
+    <row r="334" ht="18" customHeight="1" s="12">
+      <c r="I334" s="19" t="n"/>
+    </row>
+    <row r="335" ht="18" customHeight="1" s="12">
+      <c r="I335" s="19" t="n"/>
+    </row>
+    <row r="336" ht="18" customHeight="1" s="12">
+      <c r="I336" s="19" t="n"/>
+    </row>
+    <row r="337" ht="18" customHeight="1" s="12">
+      <c r="I337" s="19" t="n"/>
+    </row>
+    <row r="338" ht="18" customHeight="1" s="12">
+      <c r="I338" s="19" t="n"/>
+    </row>
+    <row r="339" ht="18" customHeight="1" s="12">
+      <c r="I339" s="19" t="n"/>
+    </row>
+    <row r="340" ht="18" customHeight="1" s="12">
+      <c r="I340" s="19" t="n"/>
+    </row>
+    <row r="341" ht="18" customHeight="1" s="12">
+      <c r="I341" s="19" t="n"/>
+    </row>
+    <row r="342" ht="18" customHeight="1" s="12">
+      <c r="I342" s="19" t="n"/>
+    </row>
+    <row r="343" ht="18" customHeight="1" s="12">
+      <c r="I343" s="19" t="n"/>
+    </row>
+    <row r="344" ht="18" customHeight="1" s="12">
+      <c r="I344" s="19" t="n"/>
+    </row>
+    <row r="345" ht="18" customHeight="1" s="12">
+      <c r="I345" s="19" t="n"/>
+    </row>
+    <row r="346" ht="18" customHeight="1" s="12">
+      <c r="I346" s="19" t="n"/>
+    </row>
+    <row r="347" ht="18" customHeight="1" s="12">
+      <c r="I347" s="19" t="n"/>
+    </row>
+    <row r="348" ht="18" customHeight="1" s="12">
+      <c r="I348" s="19" t="n"/>
+    </row>
+    <row r="349" ht="18" customHeight="1" s="12">
+      <c r="I349" s="19" t="n"/>
+    </row>
+    <row r="350" ht="18" customHeight="1" s="12">
+      <c r="I350" s="19" t="n"/>
+    </row>
+    <row r="351" ht="18" customHeight="1" s="12">
+      <c r="I351" s="19" t="n"/>
+    </row>
+    <row r="352" ht="18" customHeight="1" s="12">
+      <c r="I352" s="19" t="n"/>
+    </row>
+    <row r="353" ht="18" customHeight="1" s="12">
+      <c r="I353" s="19" t="n"/>
+    </row>
+    <row r="354" ht="18" customHeight="1" s="12">
+      <c r="I354" s="19" t="n"/>
+    </row>
+    <row r="355" ht="18" customHeight="1" s="12">
+      <c r="I355" s="19" t="n"/>
+    </row>
+    <row r="356" ht="18" customHeight="1" s="12">
+      <c r="I356" s="19" t="n"/>
+    </row>
+    <row r="357" ht="18" customHeight="1" s="12">
+      <c r="I357" s="19" t="n"/>
+    </row>
+    <row r="358" ht="18" customHeight="1" s="12">
+      <c r="I358" s="19" t="n"/>
+    </row>
+    <row r="359" ht="18" customHeight="1" s="12">
+      <c r="I359" s="19" t="n"/>
+    </row>
+    <row r="360" ht="18" customHeight="1" s="12">
+      <c r="I360" s="19" t="n"/>
+    </row>
+    <row r="361" ht="18" customHeight="1" s="12">
+      <c r="I361" s="19" t="n"/>
+    </row>
+    <row r="362" ht="18" customHeight="1" s="12">
+      <c r="I362" s="19" t="n"/>
+    </row>
+    <row r="363" ht="18" customHeight="1" s="12">
+      <c r="I363" s="19" t="n"/>
+    </row>
+    <row r="364" ht="18" customHeight="1" s="12">
+      <c r="I364" s="19" t="n"/>
+    </row>
+    <row r="365" ht="18" customHeight="1" s="12">
+      <c r="I365" s="19" t="n"/>
+    </row>
+    <row r="366" ht="18" customHeight="1" s="12">
+      <c r="I366" s="19" t="n"/>
+    </row>
+    <row r="367" ht="18" customHeight="1" s="12">
+      <c r="I367" s="19" t="n"/>
+    </row>
+    <row r="368" ht="18" customHeight="1" s="12">
+      <c r="I368" s="19" t="n"/>
+    </row>
+    <row r="369" ht="18" customHeight="1" s="12">
+      <c r="I369" s="19" t="n"/>
+    </row>
+    <row r="370" ht="18" customHeight="1" s="12">
+      <c r="I370" s="19" t="n"/>
+    </row>
+    <row r="371" ht="18" customHeight="1" s="12">
+      <c r="I371" s="19" t="n"/>
+    </row>
+    <row r="372" ht="18" customHeight="1" s="12">
+      <c r="I372" s="19" t="n"/>
+    </row>
+    <row r="373" ht="18" customHeight="1" s="12">
+      <c r="I373" s="19" t="n"/>
+    </row>
+    <row r="374" ht="18" customHeight="1" s="12">
+      <c r="I374" s="19" t="n"/>
+    </row>
+    <row r="375" ht="18" customHeight="1" s="12">
+      <c r="I375" s="19" t="n"/>
+    </row>
+    <row r="376" ht="18" customHeight="1" s="12">
+      <c r="I376" s="19" t="n"/>
+    </row>
+    <row r="377" ht="18" customHeight="1" s="12">
+      <c r="I377" s="19" t="n"/>
+    </row>
+    <row r="378" ht="18" customHeight="1" s="12">
+      <c r="I378" s="19" t="n"/>
+    </row>
+    <row r="379" ht="18" customHeight="1" s="12">
+      <c r="I379" s="19" t="n"/>
+    </row>
+    <row r="380" ht="18" customHeight="1" s="12">
+      <c r="I380" s="19" t="n"/>
+    </row>
+    <row r="381" ht="18" customHeight="1" s="12">
+      <c r="I381" s="19" t="n"/>
+    </row>
+    <row r="382" ht="18" customHeight="1" s="12">
+      <c r="I382" s="19" t="n"/>
+    </row>
+    <row r="383" ht="18" customHeight="1" s="12">
+      <c r="I383" s="19" t="n"/>
+    </row>
+    <row r="384" ht="18" customHeight="1" s="12">
+      <c r="I384" s="19" t="n"/>
+    </row>
+    <row r="385" ht="18" customHeight="1" s="12">
+      <c r="I385" s="19" t="n"/>
+    </row>
+    <row r="386" ht="18" customHeight="1" s="12">
+      <c r="I386" s="19" t="n"/>
+    </row>
+    <row r="387" ht="18" customHeight="1" s="12">
+      <c r="I387" s="19" t="n"/>
+    </row>
+    <row r="388" ht="18" customHeight="1" s="12">
+      <c r="I388" s="19" t="n"/>
+    </row>
+    <row r="389" ht="18" customHeight="1" s="12">
+      <c r="I389" s="19" t="n"/>
+    </row>
+    <row r="390" ht="18" customHeight="1" s="12">
+      <c r="I390" s="19" t="n"/>
+    </row>
+    <row r="391" ht="18" customHeight="1" s="12">
+      <c r="I391" s="19" t="n"/>
+    </row>
+    <row r="392" ht="18" customHeight="1" s="12">
+      <c r="I392" s="19" t="n"/>
+    </row>
+    <row r="393" ht="18" customHeight="1" s="12">
+      <c r="I393" s="19" t="n"/>
+    </row>
+    <row r="394" ht="18" customHeight="1" s="12">
+      <c r="I394" s="19" t="n"/>
+    </row>
+    <row r="395" ht="18" customHeight="1" s="12">
+      <c r="I395" s="19" t="n"/>
+    </row>
+    <row r="396" ht="18" customHeight="1" s="12">
+      <c r="I396" s="19" t="n"/>
+    </row>
+    <row r="397" ht="18" customHeight="1" s="12">
+      <c r="I397" s="19" t="n"/>
+    </row>
+    <row r="398" ht="18" customHeight="1" s="12">
+      <c r="I398" s="19" t="n"/>
+    </row>
+    <row r="399" ht="18" customHeight="1" s="12">
+      <c r="I399" s="19" t="n"/>
+    </row>
+    <row r="400" ht="18" customHeight="1" s="12">
+      <c r="I400" s="19" t="n"/>
+    </row>
+    <row r="401" ht="18" customHeight="1" s="12">
+      <c r="I401" s="19" t="n"/>
+    </row>
+    <row r="402" ht="18" customHeight="1" s="12">
+      <c r="I402" s="19" t="n"/>
+    </row>
+    <row r="403" ht="18" customHeight="1" s="12">
+      <c r="I403" s="19" t="n"/>
+    </row>
+    <row r="404" ht="18" customHeight="1" s="12">
+      <c r="I404" s="19" t="n"/>
+    </row>
+    <row r="405" ht="18" customHeight="1" s="12">
+      <c r="I405" s="19" t="n"/>
+    </row>
+    <row r="406" ht="18" customHeight="1" s="12">
+      <c r="I406" s="19" t="n"/>
+    </row>
+    <row r="407" ht="18" customHeight="1" s="12">
+      <c r="I407" s="19" t="n"/>
+    </row>
+    <row r="408" ht="18" customHeight="1" s="12">
+      <c r="I408" s="19" t="n"/>
+    </row>
+    <row r="409" ht="18" customHeight="1" s="12">
+      <c r="I409" s="19" t="n"/>
+    </row>
+    <row r="410" ht="18" customHeight="1" s="12">
+      <c r="I410" s="19" t="n"/>
+    </row>
+    <row r="411" ht="18" customHeight="1" s="12">
+      <c r="I411" s="19" t="n"/>
+    </row>
+    <row r="412" ht="18" customHeight="1" s="12">
+      <c r="I412" s="19" t="n"/>
+    </row>
+    <row r="413" ht="18" customHeight="1" s="12">
+      <c r="I413" s="19" t="n"/>
+    </row>
+    <row r="414" ht="18" customHeight="1" s="12">
+      <c r="I414" s="19" t="n"/>
+    </row>
+    <row r="415" ht="18" customHeight="1" s="12">
+      <c r="I415" s="19" t="n"/>
+    </row>
+    <row r="416" ht="18" customHeight="1" s="12">
+      <c r="I416" s="19" t="n"/>
+    </row>
+    <row r="417" ht="18" customHeight="1" s="12">
+      <c r="I417" s="19" t="n"/>
+    </row>
+    <row r="418" ht="18" customHeight="1" s="12">
+      <c r="I418" s="19" t="n"/>
+    </row>
+    <row r="419" ht="18" customHeight="1" s="12">
+      <c r="I419" s="19" t="n"/>
+    </row>
+    <row r="420" ht="18" customHeight="1" s="12">
+      <c r="I420" s="19" t="n"/>
+    </row>
+    <row r="421" ht="18" customHeight="1" s="12">
+      <c r="I421" s="19" t="n"/>
+    </row>
+    <row r="422" ht="18" customHeight="1" s="12">
+      <c r="I422" s="19" t="n"/>
+    </row>
+    <row r="423" ht="18" customHeight="1" s="12">
+      <c r="I423" s="19" t="n"/>
+    </row>
+    <row r="424" ht="18" customHeight="1" s="12">
+      <c r="I424" s="19" t="n"/>
+    </row>
+    <row r="425" ht="18" customHeight="1" s="12">
+      <c r="I425" s="19" t="n"/>
+    </row>
+    <row r="426" ht="18" customHeight="1" s="12">
+      <c r="I426" s="19" t="n"/>
+    </row>
+    <row r="427" ht="18" customHeight="1" s="12">
+      <c r="I427" s="19" t="n"/>
+    </row>
+    <row r="428" ht="18" customHeight="1" s="12">
+      <c r="I428" s="19" t="n"/>
+    </row>
+    <row r="429" ht="18" customHeight="1" s="12">
+      <c r="I429" s="19" t="n"/>
+    </row>
+    <row r="430" ht="18" customHeight="1" s="12">
+      <c r="I430" s="19" t="n"/>
+    </row>
+    <row r="431" ht="18" customHeight="1" s="12">
+      <c r="I431" s="19" t="n"/>
+    </row>
+    <row r="432" ht="18" customHeight="1" s="12">
+      <c r="I432" s="19" t="n"/>
+    </row>
+    <row r="433" ht="18" customHeight="1" s="12">
+      <c r="I433" s="19" t="n"/>
+    </row>
+    <row r="434" ht="18" customHeight="1" s="12">
+      <c r="I434" s="19" t="n"/>
+    </row>
+    <row r="435" ht="18" customHeight="1" s="12">
+      <c r="I435" s="19" t="n"/>
+    </row>
+    <row r="436" ht="18" customHeight="1" s="12">
+      <c r="I436" s="19" t="n"/>
+    </row>
+    <row r="437" ht="18" customHeight="1" s="12">
+      <c r="I437" s="19" t="n"/>
+    </row>
+    <row r="438" ht="18" customHeight="1" s="12">
+      <c r="I438" s="19" t="n"/>
+    </row>
+    <row r="439" ht="18" customHeight="1" s="12">
+      <c r="I439" s="19" t="n"/>
+    </row>
+    <row r="440" ht="18" customHeight="1" s="12">
+      <c r="I440" s="19" t="n"/>
+    </row>
+    <row r="441" ht="18" customHeight="1" s="12">
+      <c r="I441" s="19" t="n"/>
+    </row>
+    <row r="442" ht="18" customHeight="1" s="12">
+      <c r="I442" s="19" t="n"/>
+    </row>
+    <row r="443" ht="18" customHeight="1" s="12">
+      <c r="I443" s="19" t="n"/>
+    </row>
+    <row r="444" ht="18" customHeight="1" s="12">
+      <c r="I444" s="19" t="n"/>
+    </row>
+    <row r="445" ht="18" customHeight="1" s="12">
+      <c r="I445" s="19" t="n"/>
+    </row>
+    <row r="446" ht="18" customHeight="1" s="12">
+      <c r="I446" s="19" t="n"/>
+    </row>
+    <row r="447" ht="18" customHeight="1" s="12">
+      <c r="I447" s="19" t="n"/>
+    </row>
+    <row r="448" ht="18" customHeight="1" s="12">
+      <c r="I448" s="19" t="n"/>
+    </row>
+    <row r="449" ht="18" customHeight="1" s="12">
+      <c r="I449" s="19" t="n"/>
+    </row>
+    <row r="450" ht="18" customHeight="1" s="12">
+      <c r="I450" s="19" t="n"/>
+    </row>
+    <row r="451" ht="18" customHeight="1" s="12">
+      <c r="I451" s="19" t="n"/>
+    </row>
+    <row r="452" ht="18" customHeight="1" s="12">
+      <c r="I452" s="19" t="n"/>
+    </row>
+    <row r="453" ht="18" customHeight="1" s="12">
+      <c r="I453" s="19" t="n"/>
+    </row>
+    <row r="454" ht="18" customHeight="1" s="12">
+      <c r="I454" s="19" t="n"/>
+    </row>
+    <row r="455" ht="18" customHeight="1" s="12">
+      <c r="I455" s="19" t="n"/>
+    </row>
+    <row r="456" ht="18" customHeight="1" s="12">
+      <c r="I456" s="19" t="n"/>
+    </row>
+    <row r="457" ht="18" customHeight="1" s="12">
+      <c r="I457" s="19" t="n"/>
+    </row>
+    <row r="458" ht="18" customHeight="1" s="12">
+      <c r="I458" s="19" t="n"/>
+    </row>
+    <row r="459" ht="18" customHeight="1" s="12">
+      <c r="I459" s="19" t="n"/>
+    </row>
+    <row r="460" ht="18" customHeight="1" s="12">
+      <c r="I460" s="19" t="n"/>
+    </row>
+    <row r="461" ht="18" customHeight="1" s="12">
+      <c r="I461" s="19" t="n"/>
+    </row>
+    <row r="462" ht="18" customHeight="1" s="12">
+      <c r="I462" s="19" t="n"/>
+    </row>
+    <row r="463" ht="18" customHeight="1" s="12">
+      <c r="I463" s="19" t="n"/>
+    </row>
+    <row r="464" ht="18" customHeight="1" s="12">
+      <c r="I464" s="19" t="n"/>
+    </row>
+    <row r="465" ht="18" customHeight="1" s="12">
+      <c r="I465" s="19" t="n"/>
+    </row>
+    <row r="466" ht="18" customHeight="1" s="12">
+      <c r="I466" s="19" t="n"/>
+    </row>
+    <row r="467" ht="18" customHeight="1" s="12">
+      <c r="I467" s="19" t="n"/>
+    </row>
+    <row r="468" ht="18" customHeight="1" s="12">
+      <c r="I468" s="19" t="n"/>
+    </row>
+    <row r="469" ht="18" customHeight="1" s="12">
+      <c r="I469" s="19" t="n"/>
+    </row>
+    <row r="470" ht="18" customHeight="1" s="12">
+      <c r="I470" s="19" t="n"/>
+    </row>
+    <row r="471" ht="18" customHeight="1" s="12">
+      <c r="I471" s="19" t="n"/>
+    </row>
+    <row r="472" ht="18" customHeight="1" s="12">
+      <c r="I472" s="19" t="n"/>
+    </row>
+    <row r="473" ht="18" customHeight="1" s="12">
+      <c r="I473" s="19" t="n"/>
+    </row>
+    <row r="474" ht="18" customHeight="1" s="12">
+      <c r="I474" s="19" t="n"/>
+    </row>
+    <row r="475" ht="18" customHeight="1" s="12">
+      <c r="I475" s="19" t="n"/>
+    </row>
+    <row r="476" ht="18" customHeight="1" s="12">
+      <c r="I476" s="19" t="n"/>
+    </row>
+    <row r="477" ht="18" customHeight="1" s="12">
+      <c r="I477" s="19" t="n"/>
+    </row>
+    <row r="478" ht="18" customHeight="1" s="12">
+      <c r="I478" s="19" t="n"/>
+    </row>
+    <row r="479" ht="18" customHeight="1" s="12">
+      <c r="I479" s="19" t="n"/>
+    </row>
+    <row r="480" ht="18" customHeight="1" s="12">
+      <c r="I480" s="19" t="n"/>
+    </row>
+    <row r="481" ht="18" customHeight="1" s="12">
+      <c r="I481" s="19" t="n"/>
+    </row>
+    <row r="482" ht="18" customHeight="1" s="12">
+      <c r="I482" s="19" t="n"/>
+    </row>
+    <row r="483" ht="18" customHeight="1" s="12">
+      <c r="I483" s="19" t="n"/>
+    </row>
+    <row r="484" ht="18" customHeight="1" s="12">
+      <c r="I484" s="19" t="n"/>
+    </row>
+    <row r="485" ht="18" customHeight="1" s="12">
+      <c r="I485" s="19" t="n"/>
+    </row>
+    <row r="486" ht="18" customHeight="1" s="12">
+      <c r="I486" s="19" t="n"/>
+    </row>
+    <row r="487" ht="18" customHeight="1" s="12">
+      <c r="I487" s="19" t="n"/>
+    </row>
+    <row r="488" ht="18" customHeight="1" s="12">
+      <c r="I488" s="19" t="n"/>
+    </row>
+    <row r="489" ht="18" customHeight="1" s="12">
+      <c r="I489" s="19" t="n"/>
+    </row>
+    <row r="490" ht="18" customHeight="1" s="12">
+      <c r="I490" s="19" t="n"/>
+    </row>
+    <row r="491" ht="18" customHeight="1" s="12">
+      <c r="I491" s="19" t="n"/>
+    </row>
+    <row r="492" ht="18" customHeight="1" s="12">
+      <c r="I492" s="19" t="n"/>
+    </row>
+    <row r="493" ht="18" customHeight="1" s="12">
+      <c r="I493" s="19" t="n"/>
+    </row>
+    <row r="494" ht="18" customHeight="1" s="12">
+      <c r="I494" s="19" t="n"/>
+    </row>
+    <row r="495" ht="18" customHeight="1" s="12">
+      <c r="I495" s="19" t="n"/>
+    </row>
+    <row r="496" ht="18" customHeight="1" s="12">
+      <c r="I496" s="19" t="n"/>
+    </row>
+    <row r="497" ht="18" customHeight="1" s="12">
+      <c r="I497" s="19" t="n"/>
+    </row>
+    <row r="498" ht="18" customHeight="1" s="12">
+      <c r="I498" s="19" t="n"/>
+    </row>
+    <row r="499" ht="18" customHeight="1" s="12">
+      <c r="I499" s="19" t="n"/>
+    </row>
+    <row r="500" ht="18" customHeight="1" s="12">
+      <c r="I500" s="19" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -1406,7 +2856,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K500"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col width="20" customWidth="1" style="12" min="1" max="1"/>
@@ -1557,6 +3007,1497 @@
       </c>
       <c r="I3" s="8" t="n"/>
       <c r="J3" s="8" t="n"/>
+    </row>
+    <row r="4" ht="18" customHeight="1" s="12">
+      <c r="I4" s="19" t="n"/>
+    </row>
+    <row r="5" ht="18" customHeight="1" s="12">
+      <c r="I5" s="19" t="n"/>
+    </row>
+    <row r="6" ht="18" customHeight="1" s="12">
+      <c r="I6" s="19" t="n"/>
+    </row>
+    <row r="7" ht="18" customHeight="1" s="12">
+      <c r="I7" s="19" t="n"/>
+    </row>
+    <row r="8" ht="18" customHeight="1" s="12">
+      <c r="I8" s="19" t="n"/>
+    </row>
+    <row r="9" ht="18" customHeight="1" s="12">
+      <c r="I9" s="19" t="n"/>
+    </row>
+    <row r="10" ht="18" customHeight="1" s="12">
+      <c r="I10" s="19" t="n"/>
+    </row>
+    <row r="11" ht="18" customHeight="1" s="12">
+      <c r="I11" s="19" t="n"/>
+    </row>
+    <row r="12" ht="18" customHeight="1" s="12">
+      <c r="I12" s="19" t="n"/>
+    </row>
+    <row r="13" ht="18" customHeight="1" s="12">
+      <c r="I13" s="19" t="n"/>
+    </row>
+    <row r="14" ht="18" customHeight="1" s="12">
+      <c r="I14" s="19" t="n"/>
+    </row>
+    <row r="15" ht="18" customHeight="1" s="12">
+      <c r="I15" s="19" t="n"/>
+    </row>
+    <row r="16" ht="18" customHeight="1" s="12">
+      <c r="I16" s="19" t="n"/>
+    </row>
+    <row r="17" ht="18" customHeight="1" s="12">
+      <c r="I17" s="19" t="n"/>
+    </row>
+    <row r="18" ht="18" customHeight="1" s="12">
+      <c r="I18" s="19" t="n"/>
+    </row>
+    <row r="19" ht="18" customHeight="1" s="12">
+      <c r="I19" s="19" t="n"/>
+    </row>
+    <row r="20" ht="18" customHeight="1" s="12">
+      <c r="I20" s="19" t="n"/>
+    </row>
+    <row r="21" ht="18" customHeight="1" s="12">
+      <c r="I21" s="19" t="n"/>
+    </row>
+    <row r="22" ht="18" customHeight="1" s="12">
+      <c r="I22" s="19" t="n"/>
+    </row>
+    <row r="23" ht="18" customHeight="1" s="12">
+      <c r="I23" s="19" t="n"/>
+    </row>
+    <row r="24" ht="18" customHeight="1" s="12">
+      <c r="I24" s="19" t="n"/>
+    </row>
+    <row r="25" ht="18" customHeight="1" s="12">
+      <c r="I25" s="19" t="n"/>
+    </row>
+    <row r="26" ht="18" customHeight="1" s="12">
+      <c r="I26" s="19" t="n"/>
+    </row>
+    <row r="27" ht="18" customHeight="1" s="12">
+      <c r="I27" s="19" t="n"/>
+    </row>
+    <row r="28" ht="18" customHeight="1" s="12">
+      <c r="I28" s="19" t="n"/>
+    </row>
+    <row r="29" ht="18" customHeight="1" s="12">
+      <c r="I29" s="19" t="n"/>
+    </row>
+    <row r="30" ht="18" customHeight="1" s="12">
+      <c r="I30" s="19" t="n"/>
+    </row>
+    <row r="31" ht="18" customHeight="1" s="12">
+      <c r="I31" s="19" t="n"/>
+    </row>
+    <row r="32" ht="18" customHeight="1" s="12">
+      <c r="I32" s="19" t="n"/>
+    </row>
+    <row r="33" ht="18" customHeight="1" s="12">
+      <c r="I33" s="19" t="n"/>
+    </row>
+    <row r="34" ht="18" customHeight="1" s="12">
+      <c r="I34" s="19" t="n"/>
+    </row>
+    <row r="35" ht="18" customHeight="1" s="12">
+      <c r="I35" s="19" t="n"/>
+    </row>
+    <row r="36" ht="18" customHeight="1" s="12">
+      <c r="I36" s="19" t="n"/>
+    </row>
+    <row r="37" ht="18" customHeight="1" s="12">
+      <c r="I37" s="19" t="n"/>
+    </row>
+    <row r="38" ht="18" customHeight="1" s="12">
+      <c r="I38" s="19" t="n"/>
+    </row>
+    <row r="39" ht="18" customHeight="1" s="12">
+      <c r="I39" s="19" t="n"/>
+    </row>
+    <row r="40" ht="18" customHeight="1" s="12">
+      <c r="I40" s="19" t="n"/>
+    </row>
+    <row r="41" ht="18" customHeight="1" s="12">
+      <c r="I41" s="19" t="n"/>
+    </row>
+    <row r="42" ht="18" customHeight="1" s="12">
+      <c r="I42" s="19" t="n"/>
+    </row>
+    <row r="43" ht="18" customHeight="1" s="12">
+      <c r="I43" s="19" t="n"/>
+    </row>
+    <row r="44" ht="18" customHeight="1" s="12">
+      <c r="I44" s="19" t="n"/>
+    </row>
+    <row r="45" ht="18" customHeight="1" s="12">
+      <c r="I45" s="19" t="n"/>
+    </row>
+    <row r="46" ht="18" customHeight="1" s="12">
+      <c r="I46" s="19" t="n"/>
+    </row>
+    <row r="47" ht="18" customHeight="1" s="12">
+      <c r="I47" s="19" t="n"/>
+    </row>
+    <row r="48" ht="18" customHeight="1" s="12">
+      <c r="I48" s="19" t="n"/>
+    </row>
+    <row r="49" ht="18" customHeight="1" s="12">
+      <c r="I49" s="19" t="n"/>
+    </row>
+    <row r="50" ht="18" customHeight="1" s="12">
+      <c r="I50" s="19" t="n"/>
+    </row>
+    <row r="51" ht="18" customHeight="1" s="12">
+      <c r="I51" s="19" t="n"/>
+    </row>
+    <row r="52" ht="18" customHeight="1" s="12">
+      <c r="I52" s="19" t="n"/>
+    </row>
+    <row r="53" ht="18" customHeight="1" s="12">
+      <c r="I53" s="19" t="n"/>
+    </row>
+    <row r="54" ht="18" customHeight="1" s="12">
+      <c r="I54" s="19" t="n"/>
+    </row>
+    <row r="55" ht="18" customHeight="1" s="12">
+      <c r="I55" s="19" t="n"/>
+    </row>
+    <row r="56" ht="18" customHeight="1" s="12">
+      <c r="I56" s="19" t="n"/>
+    </row>
+    <row r="57" ht="18" customHeight="1" s="12">
+      <c r="I57" s="19" t="n"/>
+    </row>
+    <row r="58" ht="18" customHeight="1" s="12">
+      <c r="I58" s="19" t="n"/>
+    </row>
+    <row r="59" ht="18" customHeight="1" s="12">
+      <c r="I59" s="19" t="n"/>
+    </row>
+    <row r="60" ht="18" customHeight="1" s="12">
+      <c r="I60" s="19" t="n"/>
+    </row>
+    <row r="61" ht="18" customHeight="1" s="12">
+      <c r="I61" s="19" t="n"/>
+    </row>
+    <row r="62" ht="18" customHeight="1" s="12">
+      <c r="I62" s="19" t="n"/>
+    </row>
+    <row r="63" ht="18" customHeight="1" s="12">
+      <c r="I63" s="19" t="n"/>
+    </row>
+    <row r="64" ht="18" customHeight="1" s="12">
+      <c r="I64" s="19" t="n"/>
+    </row>
+    <row r="65" ht="18" customHeight="1" s="12">
+      <c r="I65" s="19" t="n"/>
+    </row>
+    <row r="66" ht="18" customHeight="1" s="12">
+      <c r="I66" s="19" t="n"/>
+    </row>
+    <row r="67" ht="18" customHeight="1" s="12">
+      <c r="I67" s="19" t="n"/>
+    </row>
+    <row r="68" ht="18" customHeight="1" s="12">
+      <c r="I68" s="19" t="n"/>
+    </row>
+    <row r="69" ht="18" customHeight="1" s="12">
+      <c r="I69" s="19" t="n"/>
+    </row>
+    <row r="70" ht="18" customHeight="1" s="12">
+      <c r="I70" s="19" t="n"/>
+    </row>
+    <row r="71" ht="18" customHeight="1" s="12">
+      <c r="I71" s="19" t="n"/>
+    </row>
+    <row r="72" ht="18" customHeight="1" s="12">
+      <c r="I72" s="19" t="n"/>
+    </row>
+    <row r="73" ht="18" customHeight="1" s="12">
+      <c r="I73" s="19" t="n"/>
+    </row>
+    <row r="74" ht="18" customHeight="1" s="12">
+      <c r="I74" s="19" t="n"/>
+    </row>
+    <row r="75" ht="18" customHeight="1" s="12">
+      <c r="I75" s="19" t="n"/>
+    </row>
+    <row r="76" ht="18" customHeight="1" s="12">
+      <c r="I76" s="19" t="n"/>
+    </row>
+    <row r="77" ht="18" customHeight="1" s="12">
+      <c r="I77" s="19" t="n"/>
+    </row>
+    <row r="78" ht="18" customHeight="1" s="12">
+      <c r="I78" s="19" t="n"/>
+    </row>
+    <row r="79" ht="18" customHeight="1" s="12">
+      <c r="I79" s="19" t="n"/>
+    </row>
+    <row r="80" ht="18" customHeight="1" s="12">
+      <c r="I80" s="19" t="n"/>
+    </row>
+    <row r="81" ht="18" customHeight="1" s="12">
+      <c r="I81" s="19" t="n"/>
+    </row>
+    <row r="82" ht="18" customHeight="1" s="12">
+      <c r="I82" s="19" t="n"/>
+    </row>
+    <row r="83" ht="18" customHeight="1" s="12">
+      <c r="I83" s="19" t="n"/>
+    </row>
+    <row r="84" ht="18" customHeight="1" s="12">
+      <c r="I84" s="19" t="n"/>
+    </row>
+    <row r="85" ht="18" customHeight="1" s="12">
+      <c r="I85" s="19" t="n"/>
+    </row>
+    <row r="86" ht="18" customHeight="1" s="12">
+      <c r="I86" s="19" t="n"/>
+    </row>
+    <row r="87" ht="18" customHeight="1" s="12">
+      <c r="I87" s="19" t="n"/>
+    </row>
+    <row r="88" ht="18" customHeight="1" s="12">
+      <c r="I88" s="19" t="n"/>
+    </row>
+    <row r="89" ht="18" customHeight="1" s="12">
+      <c r="I89" s="19" t="n"/>
+    </row>
+    <row r="90" ht="18" customHeight="1" s="12">
+      <c r="I90" s="19" t="n"/>
+    </row>
+    <row r="91" ht="18" customHeight="1" s="12">
+      <c r="I91" s="19" t="n"/>
+    </row>
+    <row r="92" ht="18" customHeight="1" s="12">
+      <c r="I92" s="19" t="n"/>
+    </row>
+    <row r="93" ht="18" customHeight="1" s="12">
+      <c r="I93" s="19" t="n"/>
+    </row>
+    <row r="94" ht="18" customHeight="1" s="12">
+      <c r="I94" s="19" t="n"/>
+    </row>
+    <row r="95" ht="18" customHeight="1" s="12">
+      <c r="I95" s="19" t="n"/>
+    </row>
+    <row r="96" ht="18" customHeight="1" s="12">
+      <c r="I96" s="19" t="n"/>
+    </row>
+    <row r="97" ht="18" customHeight="1" s="12">
+      <c r="I97" s="19" t="n"/>
+    </row>
+    <row r="98" ht="18" customHeight="1" s="12">
+      <c r="I98" s="19" t="n"/>
+    </row>
+    <row r="99" ht="18" customHeight="1" s="12">
+      <c r="I99" s="19" t="n"/>
+    </row>
+    <row r="100" ht="18" customHeight="1" s="12">
+      <c r="I100" s="19" t="n"/>
+    </row>
+    <row r="101" ht="18" customHeight="1" s="12">
+      <c r="I101" s="19" t="n"/>
+    </row>
+    <row r="102" ht="18" customHeight="1" s="12">
+      <c r="I102" s="19" t="n"/>
+    </row>
+    <row r="103" ht="18" customHeight="1" s="12">
+      <c r="I103" s="19" t="n"/>
+    </row>
+    <row r="104" ht="18" customHeight="1" s="12">
+      <c r="I104" s="19" t="n"/>
+    </row>
+    <row r="105" ht="18" customHeight="1" s="12">
+      <c r="I105" s="19" t="n"/>
+    </row>
+    <row r="106" ht="18" customHeight="1" s="12">
+      <c r="I106" s="19" t="n"/>
+    </row>
+    <row r="107" ht="18" customHeight="1" s="12">
+      <c r="I107" s="19" t="n"/>
+    </row>
+    <row r="108" ht="18" customHeight="1" s="12">
+      <c r="I108" s="19" t="n"/>
+    </row>
+    <row r="109" ht="18" customHeight="1" s="12">
+      <c r="I109" s="19" t="n"/>
+    </row>
+    <row r="110" ht="18" customHeight="1" s="12">
+      <c r="I110" s="19" t="n"/>
+    </row>
+    <row r="111" ht="18" customHeight="1" s="12">
+      <c r="I111" s="19" t="n"/>
+    </row>
+    <row r="112" ht="18" customHeight="1" s="12">
+      <c r="I112" s="19" t="n"/>
+    </row>
+    <row r="113" ht="18" customHeight="1" s="12">
+      <c r="I113" s="19" t="n"/>
+    </row>
+    <row r="114" ht="18" customHeight="1" s="12">
+      <c r="I114" s="19" t="n"/>
+    </row>
+    <row r="115" ht="18" customHeight="1" s="12">
+      <c r="I115" s="19" t="n"/>
+    </row>
+    <row r="116" ht="18" customHeight="1" s="12">
+      <c r="I116" s="19" t="n"/>
+    </row>
+    <row r="117" ht="18" customHeight="1" s="12">
+      <c r="I117" s="19" t="n"/>
+    </row>
+    <row r="118" ht="18" customHeight="1" s="12">
+      <c r="I118" s="19" t="n"/>
+    </row>
+    <row r="119" ht="18" customHeight="1" s="12">
+      <c r="I119" s="19" t="n"/>
+    </row>
+    <row r="120" ht="18" customHeight="1" s="12">
+      <c r="I120" s="19" t="n"/>
+    </row>
+    <row r="121" ht="18" customHeight="1" s="12">
+      <c r="I121" s="19" t="n"/>
+    </row>
+    <row r="122" ht="18" customHeight="1" s="12">
+      <c r="I122" s="19" t="n"/>
+    </row>
+    <row r="123" ht="18" customHeight="1" s="12">
+      <c r="I123" s="19" t="n"/>
+    </row>
+    <row r="124" ht="18" customHeight="1" s="12">
+      <c r="I124" s="19" t="n"/>
+    </row>
+    <row r="125" ht="18" customHeight="1" s="12">
+      <c r="I125" s="19" t="n"/>
+    </row>
+    <row r="126" ht="18" customHeight="1" s="12">
+      <c r="I126" s="19" t="n"/>
+    </row>
+    <row r="127" ht="18" customHeight="1" s="12">
+      <c r="I127" s="19" t="n"/>
+    </row>
+    <row r="128" ht="18" customHeight="1" s="12">
+      <c r="I128" s="19" t="n"/>
+    </row>
+    <row r="129" ht="18" customHeight="1" s="12">
+      <c r="I129" s="19" t="n"/>
+    </row>
+    <row r="130" ht="18" customHeight="1" s="12">
+      <c r="I130" s="19" t="n"/>
+    </row>
+    <row r="131" ht="18" customHeight="1" s="12">
+      <c r="I131" s="19" t="n"/>
+    </row>
+    <row r="132" ht="18" customHeight="1" s="12">
+      <c r="I132" s="19" t="n"/>
+    </row>
+    <row r="133" ht="18" customHeight="1" s="12">
+      <c r="I133" s="19" t="n"/>
+    </row>
+    <row r="134" ht="18" customHeight="1" s="12">
+      <c r="I134" s="19" t="n"/>
+    </row>
+    <row r="135" ht="18" customHeight="1" s="12">
+      <c r="I135" s="19" t="n"/>
+    </row>
+    <row r="136" ht="18" customHeight="1" s="12">
+      <c r="I136" s="19" t="n"/>
+    </row>
+    <row r="137" ht="18" customHeight="1" s="12">
+      <c r="I137" s="19" t="n"/>
+    </row>
+    <row r="138" ht="18" customHeight="1" s="12">
+      <c r="I138" s="19" t="n"/>
+    </row>
+    <row r="139" ht="18" customHeight="1" s="12">
+      <c r="I139" s="19" t="n"/>
+    </row>
+    <row r="140" ht="18" customHeight="1" s="12">
+      <c r="I140" s="19" t="n"/>
+    </row>
+    <row r="141" ht="18" customHeight="1" s="12">
+      <c r="I141" s="19" t="n"/>
+    </row>
+    <row r="142" ht="18" customHeight="1" s="12">
+      <c r="I142" s="19" t="n"/>
+    </row>
+    <row r="143" ht="18" customHeight="1" s="12">
+      <c r="I143" s="19" t="n"/>
+    </row>
+    <row r="144" ht="18" customHeight="1" s="12">
+      <c r="I144" s="19" t="n"/>
+    </row>
+    <row r="145" ht="18" customHeight="1" s="12">
+      <c r="I145" s="19" t="n"/>
+    </row>
+    <row r="146" ht="18" customHeight="1" s="12">
+      <c r="I146" s="19" t="n"/>
+    </row>
+    <row r="147" ht="18" customHeight="1" s="12">
+      <c r="I147" s="19" t="n"/>
+    </row>
+    <row r="148" ht="18" customHeight="1" s="12">
+      <c r="I148" s="19" t="n"/>
+    </row>
+    <row r="149" ht="18" customHeight="1" s="12">
+      <c r="I149" s="19" t="n"/>
+    </row>
+    <row r="150" ht="18" customHeight="1" s="12">
+      <c r="I150" s="19" t="n"/>
+    </row>
+    <row r="151" ht="18" customHeight="1" s="12">
+      <c r="I151" s="19" t="n"/>
+    </row>
+    <row r="152" ht="18" customHeight="1" s="12">
+      <c r="I152" s="19" t="n"/>
+    </row>
+    <row r="153" ht="18" customHeight="1" s="12">
+      <c r="I153" s="19" t="n"/>
+    </row>
+    <row r="154" ht="18" customHeight="1" s="12">
+      <c r="I154" s="19" t="n"/>
+    </row>
+    <row r="155" ht="18" customHeight="1" s="12">
+      <c r="I155" s="19" t="n"/>
+    </row>
+    <row r="156" ht="18" customHeight="1" s="12">
+      <c r="I156" s="19" t="n"/>
+    </row>
+    <row r="157" ht="18" customHeight="1" s="12">
+      <c r="I157" s="19" t="n"/>
+    </row>
+    <row r="158" ht="18" customHeight="1" s="12">
+      <c r="I158" s="19" t="n"/>
+    </row>
+    <row r="159" ht="18" customHeight="1" s="12">
+      <c r="I159" s="19" t="n"/>
+    </row>
+    <row r="160" ht="18" customHeight="1" s="12">
+      <c r="I160" s="19" t="n"/>
+    </row>
+    <row r="161" ht="18" customHeight="1" s="12">
+      <c r="I161" s="19" t="n"/>
+    </row>
+    <row r="162" ht="18" customHeight="1" s="12">
+      <c r="I162" s="19" t="n"/>
+    </row>
+    <row r="163" ht="18" customHeight="1" s="12">
+      <c r="I163" s="19" t="n"/>
+    </row>
+    <row r="164" ht="18" customHeight="1" s="12">
+      <c r="I164" s="19" t="n"/>
+    </row>
+    <row r="165" ht="18" customHeight="1" s="12">
+      <c r="I165" s="19" t="n"/>
+    </row>
+    <row r="166" ht="18" customHeight="1" s="12">
+      <c r="I166" s="19" t="n"/>
+    </row>
+    <row r="167" ht="18" customHeight="1" s="12">
+      <c r="I167" s="19" t="n"/>
+    </row>
+    <row r="168" ht="18" customHeight="1" s="12">
+      <c r="I168" s="19" t="n"/>
+    </row>
+    <row r="169" ht="18" customHeight="1" s="12">
+      <c r="I169" s="19" t="n"/>
+    </row>
+    <row r="170" ht="18" customHeight="1" s="12">
+      <c r="I170" s="19" t="n"/>
+    </row>
+    <row r="171" ht="18" customHeight="1" s="12">
+      <c r="I171" s="19" t="n"/>
+    </row>
+    <row r="172" ht="18" customHeight="1" s="12">
+      <c r="I172" s="19" t="n"/>
+    </row>
+    <row r="173" ht="18" customHeight="1" s="12">
+      <c r="I173" s="19" t="n"/>
+    </row>
+    <row r="174" ht="18" customHeight="1" s="12">
+      <c r="I174" s="19" t="n"/>
+    </row>
+    <row r="175" ht="18" customHeight="1" s="12">
+      <c r="I175" s="19" t="n"/>
+    </row>
+    <row r="176" ht="18" customHeight="1" s="12">
+      <c r="I176" s="19" t="n"/>
+    </row>
+    <row r="177" ht="18" customHeight="1" s="12">
+      <c r="I177" s="19" t="n"/>
+    </row>
+    <row r="178" ht="18" customHeight="1" s="12">
+      <c r="I178" s="19" t="n"/>
+    </row>
+    <row r="179" ht="18" customHeight="1" s="12">
+      <c r="I179" s="19" t="n"/>
+    </row>
+    <row r="180" ht="18" customHeight="1" s="12">
+      <c r="I180" s="19" t="n"/>
+    </row>
+    <row r="181" ht="18" customHeight="1" s="12">
+      <c r="I181" s="19" t="n"/>
+    </row>
+    <row r="182" ht="18" customHeight="1" s="12">
+      <c r="I182" s="19" t="n"/>
+    </row>
+    <row r="183" ht="18" customHeight="1" s="12">
+      <c r="I183" s="19" t="n"/>
+    </row>
+    <row r="184" ht="18" customHeight="1" s="12">
+      <c r="I184" s="19" t="n"/>
+    </row>
+    <row r="185" ht="18" customHeight="1" s="12">
+      <c r="I185" s="19" t="n"/>
+    </row>
+    <row r="186" ht="18" customHeight="1" s="12">
+      <c r="I186" s="19" t="n"/>
+    </row>
+    <row r="187" ht="18" customHeight="1" s="12">
+      <c r="I187" s="19" t="n"/>
+    </row>
+    <row r="188" ht="18" customHeight="1" s="12">
+      <c r="I188" s="19" t="n"/>
+    </row>
+    <row r="189" ht="18" customHeight="1" s="12">
+      <c r="I189" s="19" t="n"/>
+    </row>
+    <row r="190" ht="18" customHeight="1" s="12">
+      <c r="I190" s="19" t="n"/>
+    </row>
+    <row r="191" ht="18" customHeight="1" s="12">
+      <c r="I191" s="19" t="n"/>
+    </row>
+    <row r="192" ht="18" customHeight="1" s="12">
+      <c r="I192" s="19" t="n"/>
+    </row>
+    <row r="193" ht="18" customHeight="1" s="12">
+      <c r="I193" s="19" t="n"/>
+    </row>
+    <row r="194" ht="18" customHeight="1" s="12">
+      <c r="I194" s="19" t="n"/>
+    </row>
+    <row r="195" ht="18" customHeight="1" s="12">
+      <c r="I195" s="19" t="n"/>
+    </row>
+    <row r="196" ht="18" customHeight="1" s="12">
+      <c r="I196" s="19" t="n"/>
+    </row>
+    <row r="197" ht="18" customHeight="1" s="12">
+      <c r="I197" s="19" t="n"/>
+    </row>
+    <row r="198" ht="18" customHeight="1" s="12">
+      <c r="I198" s="19" t="n"/>
+    </row>
+    <row r="199" ht="18" customHeight="1" s="12">
+      <c r="I199" s="19" t="n"/>
+    </row>
+    <row r="200" ht="18" customHeight="1" s="12">
+      <c r="I200" s="19" t="n"/>
+    </row>
+    <row r="201" ht="18" customHeight="1" s="12">
+      <c r="I201" s="19" t="n"/>
+    </row>
+    <row r="202" ht="18" customHeight="1" s="12">
+      <c r="I202" s="19" t="n"/>
+    </row>
+    <row r="203" ht="18" customHeight="1" s="12">
+      <c r="I203" s="19" t="n"/>
+    </row>
+    <row r="204" ht="18" customHeight="1" s="12">
+      <c r="I204" s="19" t="n"/>
+    </row>
+    <row r="205" ht="18" customHeight="1" s="12">
+      <c r="I205" s="19" t="n"/>
+    </row>
+    <row r="206" ht="18" customHeight="1" s="12">
+      <c r="I206" s="19" t="n"/>
+    </row>
+    <row r="207" ht="18" customHeight="1" s="12">
+      <c r="I207" s="19" t="n"/>
+    </row>
+    <row r="208" ht="18" customHeight="1" s="12">
+      <c r="I208" s="19" t="n"/>
+    </row>
+    <row r="209" ht="18" customHeight="1" s="12">
+      <c r="I209" s="19" t="n"/>
+    </row>
+    <row r="210" ht="18" customHeight="1" s="12">
+      <c r="I210" s="19" t="n"/>
+    </row>
+    <row r="211" ht="18" customHeight="1" s="12">
+      <c r="I211" s="19" t="n"/>
+    </row>
+    <row r="212" ht="18" customHeight="1" s="12">
+      <c r="I212" s="19" t="n"/>
+    </row>
+    <row r="213" ht="18" customHeight="1" s="12">
+      <c r="I213" s="19" t="n"/>
+    </row>
+    <row r="214" ht="18" customHeight="1" s="12">
+      <c r="I214" s="19" t="n"/>
+    </row>
+    <row r="215" ht="18" customHeight="1" s="12">
+      <c r="I215" s="19" t="n"/>
+    </row>
+    <row r="216" ht="18" customHeight="1" s="12">
+      <c r="I216" s="19" t="n"/>
+    </row>
+    <row r="217" ht="18" customHeight="1" s="12">
+      <c r="I217" s="19" t="n"/>
+    </row>
+    <row r="218" ht="18" customHeight="1" s="12">
+      <c r="I218" s="19" t="n"/>
+    </row>
+    <row r="219" ht="18" customHeight="1" s="12">
+      <c r="I219" s="19" t="n"/>
+    </row>
+    <row r="220" ht="18" customHeight="1" s="12">
+      <c r="I220" s="19" t="n"/>
+    </row>
+    <row r="221" ht="18" customHeight="1" s="12">
+      <c r="I221" s="19" t="n"/>
+    </row>
+    <row r="222" ht="18" customHeight="1" s="12">
+      <c r="I222" s="19" t="n"/>
+    </row>
+    <row r="223" ht="18" customHeight="1" s="12">
+      <c r="I223" s="19" t="n"/>
+    </row>
+    <row r="224" ht="18" customHeight="1" s="12">
+      <c r="I224" s="19" t="n"/>
+    </row>
+    <row r="225" ht="18" customHeight="1" s="12">
+      <c r="I225" s="19" t="n"/>
+    </row>
+    <row r="226" ht="18" customHeight="1" s="12">
+      <c r="I226" s="19" t="n"/>
+    </row>
+    <row r="227" ht="18" customHeight="1" s="12">
+      <c r="I227" s="19" t="n"/>
+    </row>
+    <row r="228" ht="18" customHeight="1" s="12">
+      <c r="I228" s="19" t="n"/>
+    </row>
+    <row r="229" ht="18" customHeight="1" s="12">
+      <c r="I229" s="19" t="n"/>
+    </row>
+    <row r="230" ht="18" customHeight="1" s="12">
+      <c r="I230" s="19" t="n"/>
+    </row>
+    <row r="231" ht="18" customHeight="1" s="12">
+      <c r="I231" s="19" t="n"/>
+    </row>
+    <row r="232" ht="18" customHeight="1" s="12">
+      <c r="I232" s="19" t="n"/>
+    </row>
+    <row r="233" ht="18" customHeight="1" s="12">
+      <c r="I233" s="19" t="n"/>
+    </row>
+    <row r="234" ht="18" customHeight="1" s="12">
+      <c r="I234" s="19" t="n"/>
+    </row>
+    <row r="235" ht="18" customHeight="1" s="12">
+      <c r="I235" s="19" t="n"/>
+    </row>
+    <row r="236" ht="18" customHeight="1" s="12">
+      <c r="I236" s="19" t="n"/>
+    </row>
+    <row r="237" ht="18" customHeight="1" s="12">
+      <c r="I237" s="19" t="n"/>
+    </row>
+    <row r="238" ht="18" customHeight="1" s="12">
+      <c r="I238" s="19" t="n"/>
+    </row>
+    <row r="239" ht="18" customHeight="1" s="12">
+      <c r="I239" s="19" t="n"/>
+    </row>
+    <row r="240" ht="18" customHeight="1" s="12">
+      <c r="I240" s="19" t="n"/>
+    </row>
+    <row r="241" ht="18" customHeight="1" s="12">
+      <c r="I241" s="19" t="n"/>
+    </row>
+    <row r="242" ht="18" customHeight="1" s="12">
+      <c r="I242" s="19" t="n"/>
+    </row>
+    <row r="243" ht="18" customHeight="1" s="12">
+      <c r="I243" s="19" t="n"/>
+    </row>
+    <row r="244" ht="18" customHeight="1" s="12">
+      <c r="I244" s="19" t="n"/>
+    </row>
+    <row r="245" ht="18" customHeight="1" s="12">
+      <c r="I245" s="19" t="n"/>
+    </row>
+    <row r="246" ht="18" customHeight="1" s="12">
+      <c r="I246" s="19" t="n"/>
+    </row>
+    <row r="247" ht="18" customHeight="1" s="12">
+      <c r="I247" s="19" t="n"/>
+    </row>
+    <row r="248" ht="18" customHeight="1" s="12">
+      <c r="I248" s="19" t="n"/>
+    </row>
+    <row r="249" ht="18" customHeight="1" s="12">
+      <c r="I249" s="19" t="n"/>
+    </row>
+    <row r="250" ht="18" customHeight="1" s="12">
+      <c r="I250" s="19" t="n"/>
+    </row>
+    <row r="251" ht="18" customHeight="1" s="12">
+      <c r="I251" s="19" t="n"/>
+    </row>
+    <row r="252" ht="18" customHeight="1" s="12">
+      <c r="I252" s="19" t="n"/>
+    </row>
+    <row r="253" ht="18" customHeight="1" s="12">
+      <c r="I253" s="19" t="n"/>
+    </row>
+    <row r="254" ht="18" customHeight="1" s="12">
+      <c r="I254" s="19" t="n"/>
+    </row>
+    <row r="255" ht="18" customHeight="1" s="12">
+      <c r="I255" s="19" t="n"/>
+    </row>
+    <row r="256" ht="18" customHeight="1" s="12">
+      <c r="I256" s="19" t="n"/>
+    </row>
+    <row r="257" ht="18" customHeight="1" s="12">
+      <c r="I257" s="19" t="n"/>
+    </row>
+    <row r="258" ht="18" customHeight="1" s="12">
+      <c r="I258" s="19" t="n"/>
+    </row>
+    <row r="259" ht="18" customHeight="1" s="12">
+      <c r="I259" s="19" t="n"/>
+    </row>
+    <row r="260" ht="18" customHeight="1" s="12">
+      <c r="I260" s="19" t="n"/>
+    </row>
+    <row r="261" ht="18" customHeight="1" s="12">
+      <c r="I261" s="19" t="n"/>
+    </row>
+    <row r="262" ht="18" customHeight="1" s="12">
+      <c r="I262" s="19" t="n"/>
+    </row>
+    <row r="263" ht="18" customHeight="1" s="12">
+      <c r="I263" s="19" t="n"/>
+    </row>
+    <row r="264" ht="18" customHeight="1" s="12">
+      <c r="I264" s="19" t="n"/>
+    </row>
+    <row r="265" ht="18" customHeight="1" s="12">
+      <c r="I265" s="19" t="n"/>
+    </row>
+    <row r="266" ht="18" customHeight="1" s="12">
+      <c r="I266" s="19" t="n"/>
+    </row>
+    <row r="267" ht="18" customHeight="1" s="12">
+      <c r="I267" s="19" t="n"/>
+    </row>
+    <row r="268" ht="18" customHeight="1" s="12">
+      <c r="I268" s="19" t="n"/>
+    </row>
+    <row r="269" ht="18" customHeight="1" s="12">
+      <c r="I269" s="19" t="n"/>
+    </row>
+    <row r="270" ht="18" customHeight="1" s="12">
+      <c r="I270" s="19" t="n"/>
+    </row>
+    <row r="271" ht="18" customHeight="1" s="12">
+      <c r="I271" s="19" t="n"/>
+    </row>
+    <row r="272" ht="18" customHeight="1" s="12">
+      <c r="I272" s="19" t="n"/>
+    </row>
+    <row r="273" ht="18" customHeight="1" s="12">
+      <c r="I273" s="19" t="n"/>
+    </row>
+    <row r="274" ht="18" customHeight="1" s="12">
+      <c r="I274" s="19" t="n"/>
+    </row>
+    <row r="275" ht="18" customHeight="1" s="12">
+      <c r="I275" s="19" t="n"/>
+    </row>
+    <row r="276" ht="18" customHeight="1" s="12">
+      <c r="I276" s="19" t="n"/>
+    </row>
+    <row r="277" ht="18" customHeight="1" s="12">
+      <c r="I277" s="19" t="n"/>
+    </row>
+    <row r="278" ht="18" customHeight="1" s="12">
+      <c r="I278" s="19" t="n"/>
+    </row>
+    <row r="279" ht="18" customHeight="1" s="12">
+      <c r="I279" s="19" t="n"/>
+    </row>
+    <row r="280" ht="18" customHeight="1" s="12">
+      <c r="I280" s="19" t="n"/>
+    </row>
+    <row r="281" ht="18" customHeight="1" s="12">
+      <c r="I281" s="19" t="n"/>
+    </row>
+    <row r="282" ht="18" customHeight="1" s="12">
+      <c r="I282" s="19" t="n"/>
+    </row>
+    <row r="283" ht="18" customHeight="1" s="12">
+      <c r="I283" s="19" t="n"/>
+    </row>
+    <row r="284" ht="18" customHeight="1" s="12">
+      <c r="I284" s="19" t="n"/>
+    </row>
+    <row r="285" ht="18" customHeight="1" s="12">
+      <c r="I285" s="19" t="n"/>
+    </row>
+    <row r="286" ht="18" customHeight="1" s="12">
+      <c r="I286" s="19" t="n"/>
+    </row>
+    <row r="287" ht="18" customHeight="1" s="12">
+      <c r="I287" s="19" t="n"/>
+    </row>
+    <row r="288" ht="18" customHeight="1" s="12">
+      <c r="I288" s="19" t="n"/>
+    </row>
+    <row r="289" ht="18" customHeight="1" s="12">
+      <c r="I289" s="19" t="n"/>
+    </row>
+    <row r="290" ht="18" customHeight="1" s="12">
+      <c r="I290" s="19" t="n"/>
+    </row>
+    <row r="291" ht="18" customHeight="1" s="12">
+      <c r="I291" s="19" t="n"/>
+    </row>
+    <row r="292" ht="18" customHeight="1" s="12">
+      <c r="I292" s="19" t="n"/>
+    </row>
+    <row r="293" ht="18" customHeight="1" s="12">
+      <c r="I293" s="19" t="n"/>
+    </row>
+    <row r="294" ht="18" customHeight="1" s="12">
+      <c r="I294" s="19" t="n"/>
+    </row>
+    <row r="295" ht="18" customHeight="1" s="12">
+      <c r="I295" s="19" t="n"/>
+    </row>
+    <row r="296" ht="18" customHeight="1" s="12">
+      <c r="I296" s="19" t="n"/>
+    </row>
+    <row r="297" ht="18" customHeight="1" s="12">
+      <c r="I297" s="19" t="n"/>
+    </row>
+    <row r="298" ht="18" customHeight="1" s="12">
+      <c r="I298" s="19" t="n"/>
+    </row>
+    <row r="299" ht="18" customHeight="1" s="12">
+      <c r="I299" s="19" t="n"/>
+    </row>
+    <row r="300" ht="18" customHeight="1" s="12">
+      <c r="I300" s="19" t="n"/>
+    </row>
+    <row r="301" ht="18" customHeight="1" s="12">
+      <c r="I301" s="19" t="n"/>
+    </row>
+    <row r="302" ht="18" customHeight="1" s="12">
+      <c r="I302" s="19" t="n"/>
+    </row>
+    <row r="303" ht="18" customHeight="1" s="12">
+      <c r="I303" s="19" t="n"/>
+    </row>
+    <row r="304" ht="18" customHeight="1" s="12">
+      <c r="I304" s="19" t="n"/>
+    </row>
+    <row r="305" ht="18" customHeight="1" s="12">
+      <c r="I305" s="19" t="n"/>
+    </row>
+    <row r="306" ht="18" customHeight="1" s="12">
+      <c r="I306" s="19" t="n"/>
+    </row>
+    <row r="307" ht="18" customHeight="1" s="12">
+      <c r="I307" s="19" t="n"/>
+    </row>
+    <row r="308" ht="18" customHeight="1" s="12">
+      <c r="I308" s="19" t="n"/>
+    </row>
+    <row r="309" ht="18" customHeight="1" s="12">
+      <c r="I309" s="19" t="n"/>
+    </row>
+    <row r="310" ht="18" customHeight="1" s="12">
+      <c r="I310" s="19" t="n"/>
+    </row>
+    <row r="311" ht="18" customHeight="1" s="12">
+      <c r="I311" s="19" t="n"/>
+    </row>
+    <row r="312" ht="18" customHeight="1" s="12">
+      <c r="I312" s="19" t="n"/>
+    </row>
+    <row r="313" ht="18" customHeight="1" s="12">
+      <c r="I313" s="19" t="n"/>
+    </row>
+    <row r="314" ht="18" customHeight="1" s="12">
+      <c r="I314" s="19" t="n"/>
+    </row>
+    <row r="315" ht="18" customHeight="1" s="12">
+      <c r="I315" s="19" t="n"/>
+    </row>
+    <row r="316" ht="18" customHeight="1" s="12">
+      <c r="I316" s="19" t="n"/>
+    </row>
+    <row r="317" ht="18" customHeight="1" s="12">
+      <c r="I317" s="19" t="n"/>
+    </row>
+    <row r="318" ht="18" customHeight="1" s="12">
+      <c r="I318" s="19" t="n"/>
+    </row>
+    <row r="319" ht="18" customHeight="1" s="12">
+      <c r="I319" s="19" t="n"/>
+    </row>
+    <row r="320" ht="18" customHeight="1" s="12">
+      <c r="I320" s="19" t="n"/>
+    </row>
+    <row r="321" ht="18" customHeight="1" s="12">
+      <c r="I321" s="19" t="n"/>
+    </row>
+    <row r="322" ht="18" customHeight="1" s="12">
+      <c r="I322" s="19" t="n"/>
+    </row>
+    <row r="323" ht="18" customHeight="1" s="12">
+      <c r="I323" s="19" t="n"/>
+    </row>
+    <row r="324" ht="18" customHeight="1" s="12">
+      <c r="I324" s="19" t="n"/>
+    </row>
+    <row r="325" ht="18" customHeight="1" s="12">
+      <c r="I325" s="19" t="n"/>
+    </row>
+    <row r="326" ht="18" customHeight="1" s="12">
+      <c r="I326" s="19" t="n"/>
+    </row>
+    <row r="327" ht="18" customHeight="1" s="12">
+      <c r="I327" s="19" t="n"/>
+    </row>
+    <row r="328" ht="18" customHeight="1" s="12">
+      <c r="I328" s="19" t="n"/>
+    </row>
+    <row r="329" ht="18" customHeight="1" s="12">
+      <c r="I329" s="19" t="n"/>
+    </row>
+    <row r="330" ht="18" customHeight="1" s="12">
+      <c r="I330" s="19" t="n"/>
+    </row>
+    <row r="331" ht="18" customHeight="1" s="12">
+      <c r="I331" s="19" t="n"/>
+    </row>
+    <row r="332" ht="18" customHeight="1" s="12">
+      <c r="I332" s="19" t="n"/>
+    </row>
+    <row r="333" ht="18" customHeight="1" s="12">
+      <c r="I333" s="19" t="n"/>
+    </row>
+    <row r="334" ht="18" customHeight="1" s="12">
+      <c r="I334" s="19" t="n"/>
+    </row>
+    <row r="335" ht="18" customHeight="1" s="12">
+      <c r="I335" s="19" t="n"/>
+    </row>
+    <row r="336" ht="18" customHeight="1" s="12">
+      <c r="I336" s="19" t="n"/>
+    </row>
+    <row r="337" ht="18" customHeight="1" s="12">
+      <c r="I337" s="19" t="n"/>
+    </row>
+    <row r="338" ht="18" customHeight="1" s="12">
+      <c r="I338" s="19" t="n"/>
+    </row>
+    <row r="339" ht="18" customHeight="1" s="12">
+      <c r="I339" s="19" t="n"/>
+    </row>
+    <row r="340" ht="18" customHeight="1" s="12">
+      <c r="I340" s="19" t="n"/>
+    </row>
+    <row r="341" ht="18" customHeight="1" s="12">
+      <c r="I341" s="19" t="n"/>
+    </row>
+    <row r="342" ht="18" customHeight="1" s="12">
+      <c r="I342" s="19" t="n"/>
+    </row>
+    <row r="343" ht="18" customHeight="1" s="12">
+      <c r="I343" s="19" t="n"/>
+    </row>
+    <row r="344" ht="18" customHeight="1" s="12">
+      <c r="I344" s="19" t="n"/>
+    </row>
+    <row r="345" ht="18" customHeight="1" s="12">
+      <c r="I345" s="19" t="n"/>
+    </row>
+    <row r="346" ht="18" customHeight="1" s="12">
+      <c r="I346" s="19" t="n"/>
+    </row>
+    <row r="347" ht="18" customHeight="1" s="12">
+      <c r="I347" s="19" t="n"/>
+    </row>
+    <row r="348" ht="18" customHeight="1" s="12">
+      <c r="I348" s="19" t="n"/>
+    </row>
+    <row r="349" ht="18" customHeight="1" s="12">
+      <c r="I349" s="19" t="n"/>
+    </row>
+    <row r="350" ht="18" customHeight="1" s="12">
+      <c r="I350" s="19" t="n"/>
+    </row>
+    <row r="351" ht="18" customHeight="1" s="12">
+      <c r="I351" s="19" t="n"/>
+    </row>
+    <row r="352" ht="18" customHeight="1" s="12">
+      <c r="I352" s="19" t="n"/>
+    </row>
+    <row r="353" ht="18" customHeight="1" s="12">
+      <c r="I353" s="19" t="n"/>
+    </row>
+    <row r="354" ht="18" customHeight="1" s="12">
+      <c r="I354" s="19" t="n"/>
+    </row>
+    <row r="355" ht="18" customHeight="1" s="12">
+      <c r="I355" s="19" t="n"/>
+    </row>
+    <row r="356" ht="18" customHeight="1" s="12">
+      <c r="I356" s="19" t="n"/>
+    </row>
+    <row r="357" ht="18" customHeight="1" s="12">
+      <c r="I357" s="19" t="n"/>
+    </row>
+    <row r="358" ht="18" customHeight="1" s="12">
+      <c r="I358" s="19" t="n"/>
+    </row>
+    <row r="359" ht="18" customHeight="1" s="12">
+      <c r="I359" s="19" t="n"/>
+    </row>
+    <row r="360" ht="18" customHeight="1" s="12">
+      <c r="I360" s="19" t="n"/>
+    </row>
+    <row r="361" ht="18" customHeight="1" s="12">
+      <c r="I361" s="19" t="n"/>
+    </row>
+    <row r="362" ht="18" customHeight="1" s="12">
+      <c r="I362" s="19" t="n"/>
+    </row>
+    <row r="363" ht="18" customHeight="1" s="12">
+      <c r="I363" s="19" t="n"/>
+    </row>
+    <row r="364" ht="18" customHeight="1" s="12">
+      <c r="I364" s="19" t="n"/>
+    </row>
+    <row r="365" ht="18" customHeight="1" s="12">
+      <c r="I365" s="19" t="n"/>
+    </row>
+    <row r="366" ht="18" customHeight="1" s="12">
+      <c r="I366" s="19" t="n"/>
+    </row>
+    <row r="367" ht="18" customHeight="1" s="12">
+      <c r="I367" s="19" t="n"/>
+    </row>
+    <row r="368" ht="18" customHeight="1" s="12">
+      <c r="I368" s="19" t="n"/>
+    </row>
+    <row r="369" ht="18" customHeight="1" s="12">
+      <c r="I369" s="19" t="n"/>
+    </row>
+    <row r="370" ht="18" customHeight="1" s="12">
+      <c r="I370" s="19" t="n"/>
+    </row>
+    <row r="371" ht="18" customHeight="1" s="12">
+      <c r="I371" s="19" t="n"/>
+    </row>
+    <row r="372" ht="18" customHeight="1" s="12">
+      <c r="I372" s="19" t="n"/>
+    </row>
+    <row r="373" ht="18" customHeight="1" s="12">
+      <c r="I373" s="19" t="n"/>
+    </row>
+    <row r="374" ht="18" customHeight="1" s="12">
+      <c r="I374" s="19" t="n"/>
+    </row>
+    <row r="375" ht="18" customHeight="1" s="12">
+      <c r="I375" s="19" t="n"/>
+    </row>
+    <row r="376" ht="18" customHeight="1" s="12">
+      <c r="I376" s="19" t="n"/>
+    </row>
+    <row r="377" ht="18" customHeight="1" s="12">
+      <c r="I377" s="19" t="n"/>
+    </row>
+    <row r="378" ht="18" customHeight="1" s="12">
+      <c r="I378" s="19" t="n"/>
+    </row>
+    <row r="379" ht="18" customHeight="1" s="12">
+      <c r="I379" s="19" t="n"/>
+    </row>
+    <row r="380" ht="18" customHeight="1" s="12">
+      <c r="I380" s="19" t="n"/>
+    </row>
+    <row r="381" ht="18" customHeight="1" s="12">
+      <c r="I381" s="19" t="n"/>
+    </row>
+    <row r="382" ht="18" customHeight="1" s="12">
+      <c r="I382" s="19" t="n"/>
+    </row>
+    <row r="383" ht="18" customHeight="1" s="12">
+      <c r="I383" s="19" t="n"/>
+    </row>
+    <row r="384" ht="18" customHeight="1" s="12">
+      <c r="I384" s="19" t="n"/>
+    </row>
+    <row r="385" ht="18" customHeight="1" s="12">
+      <c r="I385" s="19" t="n"/>
+    </row>
+    <row r="386" ht="18" customHeight="1" s="12">
+      <c r="I386" s="19" t="n"/>
+    </row>
+    <row r="387" ht="18" customHeight="1" s="12">
+      <c r="I387" s="19" t="n"/>
+    </row>
+    <row r="388" ht="18" customHeight="1" s="12">
+      <c r="I388" s="19" t="n"/>
+    </row>
+    <row r="389" ht="18" customHeight="1" s="12">
+      <c r="I389" s="19" t="n"/>
+    </row>
+    <row r="390" ht="18" customHeight="1" s="12">
+      <c r="I390" s="19" t="n"/>
+    </row>
+    <row r="391" ht="18" customHeight="1" s="12">
+      <c r="I391" s="19" t="n"/>
+    </row>
+    <row r="392" ht="18" customHeight="1" s="12">
+      <c r="I392" s="19" t="n"/>
+    </row>
+    <row r="393" ht="18" customHeight="1" s="12">
+      <c r="I393" s="19" t="n"/>
+    </row>
+    <row r="394" ht="18" customHeight="1" s="12">
+      <c r="I394" s="19" t="n"/>
+    </row>
+    <row r="395" ht="18" customHeight="1" s="12">
+      <c r="I395" s="19" t="n"/>
+    </row>
+    <row r="396" ht="18" customHeight="1" s="12">
+      <c r="I396" s="19" t="n"/>
+    </row>
+    <row r="397" ht="18" customHeight="1" s="12">
+      <c r="I397" s="19" t="n"/>
+    </row>
+    <row r="398" ht="18" customHeight="1" s="12">
+      <c r="I398" s="19" t="n"/>
+    </row>
+    <row r="399" ht="18" customHeight="1" s="12">
+      <c r="I399" s="19" t="n"/>
+    </row>
+    <row r="400" ht="18" customHeight="1" s="12">
+      <c r="I400" s="19" t="n"/>
+    </row>
+    <row r="401" ht="18" customHeight="1" s="12">
+      <c r="I401" s="19" t="n"/>
+    </row>
+    <row r="402" ht="18" customHeight="1" s="12">
+      <c r="I402" s="19" t="n"/>
+    </row>
+    <row r="403" ht="18" customHeight="1" s="12">
+      <c r="I403" s="19" t="n"/>
+    </row>
+    <row r="404" ht="18" customHeight="1" s="12">
+      <c r="I404" s="19" t="n"/>
+    </row>
+    <row r="405" ht="18" customHeight="1" s="12">
+      <c r="I405" s="19" t="n"/>
+    </row>
+    <row r="406" ht="18" customHeight="1" s="12">
+      <c r="I406" s="19" t="n"/>
+    </row>
+    <row r="407" ht="18" customHeight="1" s="12">
+      <c r="I407" s="19" t="n"/>
+    </row>
+    <row r="408" ht="18" customHeight="1" s="12">
+      <c r="I408" s="19" t="n"/>
+    </row>
+    <row r="409" ht="18" customHeight="1" s="12">
+      <c r="I409" s="19" t="n"/>
+    </row>
+    <row r="410" ht="18" customHeight="1" s="12">
+      <c r="I410" s="19" t="n"/>
+    </row>
+    <row r="411" ht="18" customHeight="1" s="12">
+      <c r="I411" s="19" t="n"/>
+    </row>
+    <row r="412" ht="18" customHeight="1" s="12">
+      <c r="I412" s="19" t="n"/>
+    </row>
+    <row r="413" ht="18" customHeight="1" s="12">
+      <c r="I413" s="19" t="n"/>
+    </row>
+    <row r="414" ht="18" customHeight="1" s="12">
+      <c r="I414" s="19" t="n"/>
+    </row>
+    <row r="415" ht="18" customHeight="1" s="12">
+      <c r="I415" s="19" t="n"/>
+    </row>
+    <row r="416" ht="18" customHeight="1" s="12">
+      <c r="I416" s="19" t="n"/>
+    </row>
+    <row r="417" ht="18" customHeight="1" s="12">
+      <c r="I417" s="19" t="n"/>
+    </row>
+    <row r="418" ht="18" customHeight="1" s="12">
+      <c r="I418" s="19" t="n"/>
+    </row>
+    <row r="419" ht="18" customHeight="1" s="12">
+      <c r="I419" s="19" t="n"/>
+    </row>
+    <row r="420" ht="18" customHeight="1" s="12">
+      <c r="I420" s="19" t="n"/>
+    </row>
+    <row r="421" ht="18" customHeight="1" s="12">
+      <c r="I421" s="19" t="n"/>
+    </row>
+    <row r="422" ht="18" customHeight="1" s="12">
+      <c r="I422" s="19" t="n"/>
+    </row>
+    <row r="423" ht="18" customHeight="1" s="12">
+      <c r="I423" s="19" t="n"/>
+    </row>
+    <row r="424" ht="18" customHeight="1" s="12">
+      <c r="I424" s="19" t="n"/>
+    </row>
+    <row r="425" ht="18" customHeight="1" s="12">
+      <c r="I425" s="19" t="n"/>
+    </row>
+    <row r="426" ht="18" customHeight="1" s="12">
+      <c r="I426" s="19" t="n"/>
+    </row>
+    <row r="427" ht="18" customHeight="1" s="12">
+      <c r="I427" s="19" t="n"/>
+    </row>
+    <row r="428" ht="18" customHeight="1" s="12">
+      <c r="I428" s="19" t="n"/>
+    </row>
+    <row r="429" ht="18" customHeight="1" s="12">
+      <c r="I429" s="19" t="n"/>
+    </row>
+    <row r="430" ht="18" customHeight="1" s="12">
+      <c r="I430" s="19" t="n"/>
+    </row>
+    <row r="431" ht="18" customHeight="1" s="12">
+      <c r="I431" s="19" t="n"/>
+    </row>
+    <row r="432" ht="18" customHeight="1" s="12">
+      <c r="I432" s="19" t="n"/>
+    </row>
+    <row r="433" ht="18" customHeight="1" s="12">
+      <c r="I433" s="19" t="n"/>
+    </row>
+    <row r="434" ht="18" customHeight="1" s="12">
+      <c r="I434" s="19" t="n"/>
+    </row>
+    <row r="435" ht="18" customHeight="1" s="12">
+      <c r="I435" s="19" t="n"/>
+    </row>
+    <row r="436" ht="18" customHeight="1" s="12">
+      <c r="I436" s="19" t="n"/>
+    </row>
+    <row r="437" ht="18" customHeight="1" s="12">
+      <c r="I437" s="19" t="n"/>
+    </row>
+    <row r="438" ht="18" customHeight="1" s="12">
+      <c r="I438" s="19" t="n"/>
+    </row>
+    <row r="439" ht="18" customHeight="1" s="12">
+      <c r="I439" s="19" t="n"/>
+    </row>
+    <row r="440" ht="18" customHeight="1" s="12">
+      <c r="I440" s="19" t="n"/>
+    </row>
+    <row r="441" ht="18" customHeight="1" s="12">
+      <c r="I441" s="19" t="n"/>
+    </row>
+    <row r="442" ht="18" customHeight="1" s="12">
+      <c r="I442" s="19" t="n"/>
+    </row>
+    <row r="443" ht="18" customHeight="1" s="12">
+      <c r="I443" s="19" t="n"/>
+    </row>
+    <row r="444" ht="18" customHeight="1" s="12">
+      <c r="I444" s="19" t="n"/>
+    </row>
+    <row r="445" ht="18" customHeight="1" s="12">
+      <c r="I445" s="19" t="n"/>
+    </row>
+    <row r="446" ht="18" customHeight="1" s="12">
+      <c r="I446" s="19" t="n"/>
+    </row>
+    <row r="447" ht="18" customHeight="1" s="12">
+      <c r="I447" s="19" t="n"/>
+    </row>
+    <row r="448" ht="18" customHeight="1" s="12">
+      <c r="I448" s="19" t="n"/>
+    </row>
+    <row r="449" ht="18" customHeight="1" s="12">
+      <c r="I449" s="19" t="n"/>
+    </row>
+    <row r="450" ht="18" customHeight="1" s="12">
+      <c r="I450" s="19" t="n"/>
+    </row>
+    <row r="451" ht="18" customHeight="1" s="12">
+      <c r="I451" s="19" t="n"/>
+    </row>
+    <row r="452" ht="18" customHeight="1" s="12">
+      <c r="I452" s="19" t="n"/>
+    </row>
+    <row r="453" ht="18" customHeight="1" s="12">
+      <c r="I453" s="19" t="n"/>
+    </row>
+    <row r="454" ht="18" customHeight="1" s="12">
+      <c r="I454" s="19" t="n"/>
+    </row>
+    <row r="455" ht="18" customHeight="1" s="12">
+      <c r="I455" s="19" t="n"/>
+    </row>
+    <row r="456" ht="18" customHeight="1" s="12">
+      <c r="I456" s="19" t="n"/>
+    </row>
+    <row r="457" ht="18" customHeight="1" s="12">
+      <c r="I457" s="19" t="n"/>
+    </row>
+    <row r="458" ht="18" customHeight="1" s="12">
+      <c r="I458" s="19" t="n"/>
+    </row>
+    <row r="459" ht="18" customHeight="1" s="12">
+      <c r="I459" s="19" t="n"/>
+    </row>
+    <row r="460" ht="18" customHeight="1" s="12">
+      <c r="I460" s="19" t="n"/>
+    </row>
+    <row r="461" ht="18" customHeight="1" s="12">
+      <c r="I461" s="19" t="n"/>
+    </row>
+    <row r="462" ht="18" customHeight="1" s="12">
+      <c r="I462" s="19" t="n"/>
+    </row>
+    <row r="463" ht="18" customHeight="1" s="12">
+      <c r="I463" s="19" t="n"/>
+    </row>
+    <row r="464" ht="18" customHeight="1" s="12">
+      <c r="I464" s="19" t="n"/>
+    </row>
+    <row r="465" ht="18" customHeight="1" s="12">
+      <c r="I465" s="19" t="n"/>
+    </row>
+    <row r="466" ht="18" customHeight="1" s="12">
+      <c r="I466" s="19" t="n"/>
+    </row>
+    <row r="467" ht="18" customHeight="1" s="12">
+      <c r="I467" s="19" t="n"/>
+    </row>
+    <row r="468" ht="18" customHeight="1" s="12">
+      <c r="I468" s="19" t="n"/>
+    </row>
+    <row r="469" ht="18" customHeight="1" s="12">
+      <c r="I469" s="19" t="n"/>
+    </row>
+    <row r="470" ht="18" customHeight="1" s="12">
+      <c r="I470" s="19" t="n"/>
+    </row>
+    <row r="471" ht="18" customHeight="1" s="12">
+      <c r="I471" s="19" t="n"/>
+    </row>
+    <row r="472" ht="18" customHeight="1" s="12">
+      <c r="I472" s="19" t="n"/>
+    </row>
+    <row r="473" ht="18" customHeight="1" s="12">
+      <c r="I473" s="19" t="n"/>
+    </row>
+    <row r="474" ht="18" customHeight="1" s="12">
+      <c r="I474" s="19" t="n"/>
+    </row>
+    <row r="475" ht="18" customHeight="1" s="12">
+      <c r="I475" s="19" t="n"/>
+    </row>
+    <row r="476" ht="18" customHeight="1" s="12">
+      <c r="I476" s="19" t="n"/>
+    </row>
+    <row r="477" ht="18" customHeight="1" s="12">
+      <c r="I477" s="19" t="n"/>
+    </row>
+    <row r="478" ht="18" customHeight="1" s="12">
+      <c r="I478" s="19" t="n"/>
+    </row>
+    <row r="479" ht="18" customHeight="1" s="12">
+      <c r="I479" s="19" t="n"/>
+    </row>
+    <row r="480" ht="18" customHeight="1" s="12">
+      <c r="I480" s="19" t="n"/>
+    </row>
+    <row r="481" ht="18" customHeight="1" s="12">
+      <c r="I481" s="19" t="n"/>
+    </row>
+    <row r="482" ht="18" customHeight="1" s="12">
+      <c r="I482" s="19" t="n"/>
+    </row>
+    <row r="483" ht="18" customHeight="1" s="12">
+      <c r="I483" s="19" t="n"/>
+    </row>
+    <row r="484" ht="18" customHeight="1" s="12">
+      <c r="I484" s="19" t="n"/>
+    </row>
+    <row r="485" ht="18" customHeight="1" s="12">
+      <c r="I485" s="19" t="n"/>
+    </row>
+    <row r="486" ht="18" customHeight="1" s="12">
+      <c r="I486" s="19" t="n"/>
+    </row>
+    <row r="487" ht="18" customHeight="1" s="12">
+      <c r="I487" s="19" t="n"/>
+    </row>
+    <row r="488" ht="18" customHeight="1" s="12">
+      <c r="I488" s="19" t="n"/>
+    </row>
+    <row r="489" ht="18" customHeight="1" s="12">
+      <c r="I489" s="19" t="n"/>
+    </row>
+    <row r="490" ht="18" customHeight="1" s="12">
+      <c r="I490" s="19" t="n"/>
+    </row>
+    <row r="491" ht="18" customHeight="1" s="12">
+      <c r="I491" s="19" t="n"/>
+    </row>
+    <row r="492" ht="18" customHeight="1" s="12">
+      <c r="I492" s="19" t="n"/>
+    </row>
+    <row r="493" ht="18" customHeight="1" s="12">
+      <c r="I493" s="19" t="n"/>
+    </row>
+    <row r="494" ht="18" customHeight="1" s="12">
+      <c r="I494" s="19" t="n"/>
+    </row>
+    <row r="495" ht="18" customHeight="1" s="12">
+      <c r="I495" s="19" t="n"/>
+    </row>
+    <row r="496" ht="18" customHeight="1" s="12">
+      <c r="I496" s="19" t="n"/>
+    </row>
+    <row r="497" ht="18" customHeight="1" s="12">
+      <c r="I497" s="19" t="n"/>
+    </row>
+    <row r="498" ht="18" customHeight="1" s="12">
+      <c r="I498" s="19" t="n"/>
+    </row>
+    <row r="499" ht="18" customHeight="1" s="12">
+      <c r="I499" s="19" t="n"/>
+    </row>
+    <row r="500" ht="18" customHeight="1" s="12">
+      <c r="I500" s="19" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -1579,7 +4520,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K500"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col width="20" customWidth="1" style="12" min="1" max="1"/>
@@ -1731,6 +4672,1497 @@
       <c r="I3" s="8" t="n"/>
       <c r="J3" s="8" t="n"/>
     </row>
+    <row r="4" ht="18" customHeight="1" s="12">
+      <c r="I4" s="19" t="n"/>
+    </row>
+    <row r="5" ht="18" customHeight="1" s="12">
+      <c r="I5" s="19" t="n"/>
+    </row>
+    <row r="6" ht="18" customHeight="1" s="12">
+      <c r="I6" s="19" t="n"/>
+    </row>
+    <row r="7" ht="18" customHeight="1" s="12">
+      <c r="I7" s="19" t="n"/>
+    </row>
+    <row r="8" ht="18" customHeight="1" s="12">
+      <c r="I8" s="19" t="n"/>
+    </row>
+    <row r="9" ht="18" customHeight="1" s="12">
+      <c r="I9" s="19" t="n"/>
+    </row>
+    <row r="10" ht="18" customHeight="1" s="12">
+      <c r="I10" s="19" t="n"/>
+    </row>
+    <row r="11" ht="18" customHeight="1" s="12">
+      <c r="I11" s="19" t="n"/>
+    </row>
+    <row r="12" ht="18" customHeight="1" s="12">
+      <c r="I12" s="19" t="n"/>
+    </row>
+    <row r="13" ht="18" customHeight="1" s="12">
+      <c r="I13" s="19" t="n"/>
+    </row>
+    <row r="14" ht="18" customHeight="1" s="12">
+      <c r="I14" s="19" t="n"/>
+    </row>
+    <row r="15" ht="18" customHeight="1" s="12">
+      <c r="I15" s="19" t="n"/>
+    </row>
+    <row r="16" ht="18" customHeight="1" s="12">
+      <c r="I16" s="19" t="n"/>
+    </row>
+    <row r="17" ht="18" customHeight="1" s="12">
+      <c r="I17" s="19" t="n"/>
+    </row>
+    <row r="18" ht="18" customHeight="1" s="12">
+      <c r="I18" s="19" t="n"/>
+    </row>
+    <row r="19" ht="18" customHeight="1" s="12">
+      <c r="I19" s="19" t="n"/>
+    </row>
+    <row r="20" ht="18" customHeight="1" s="12">
+      <c r="I20" s="19" t="n"/>
+    </row>
+    <row r="21" ht="18" customHeight="1" s="12">
+      <c r="I21" s="19" t="n"/>
+    </row>
+    <row r="22" ht="18" customHeight="1" s="12">
+      <c r="I22" s="19" t="n"/>
+    </row>
+    <row r="23" ht="18" customHeight="1" s="12">
+      <c r="I23" s="19" t="n"/>
+    </row>
+    <row r="24" ht="18" customHeight="1" s="12">
+      <c r="I24" s="19" t="n"/>
+    </row>
+    <row r="25" ht="18" customHeight="1" s="12">
+      <c r="I25" s="19" t="n"/>
+    </row>
+    <row r="26" ht="18" customHeight="1" s="12">
+      <c r="I26" s="19" t="n"/>
+    </row>
+    <row r="27" ht="18" customHeight="1" s="12">
+      <c r="I27" s="19" t="n"/>
+    </row>
+    <row r="28" ht="18" customHeight="1" s="12">
+      <c r="I28" s="19" t="n"/>
+    </row>
+    <row r="29" ht="18" customHeight="1" s="12">
+      <c r="I29" s="19" t="n"/>
+    </row>
+    <row r="30" ht="18" customHeight="1" s="12">
+      <c r="I30" s="19" t="n"/>
+    </row>
+    <row r="31" ht="18" customHeight="1" s="12">
+      <c r="I31" s="19" t="n"/>
+    </row>
+    <row r="32" ht="18" customHeight="1" s="12">
+      <c r="I32" s="19" t="n"/>
+    </row>
+    <row r="33" ht="18" customHeight="1" s="12">
+      <c r="I33" s="19" t="n"/>
+    </row>
+    <row r="34" ht="18" customHeight="1" s="12">
+      <c r="I34" s="19" t="n"/>
+    </row>
+    <row r="35" ht="18" customHeight="1" s="12">
+      <c r="I35" s="19" t="n"/>
+    </row>
+    <row r="36" ht="18" customHeight="1" s="12">
+      <c r="I36" s="19" t="n"/>
+    </row>
+    <row r="37" ht="18" customHeight="1" s="12">
+      <c r="I37" s="19" t="n"/>
+    </row>
+    <row r="38" ht="18" customHeight="1" s="12">
+      <c r="I38" s="19" t="n"/>
+    </row>
+    <row r="39" ht="18" customHeight="1" s="12">
+      <c r="I39" s="19" t="n"/>
+    </row>
+    <row r="40" ht="18" customHeight="1" s="12">
+      <c r="I40" s="19" t="n"/>
+    </row>
+    <row r="41" ht="18" customHeight="1" s="12">
+      <c r="I41" s="19" t="n"/>
+    </row>
+    <row r="42" ht="18" customHeight="1" s="12">
+      <c r="I42" s="19" t="n"/>
+    </row>
+    <row r="43" ht="18" customHeight="1" s="12">
+      <c r="I43" s="19" t="n"/>
+    </row>
+    <row r="44" ht="18" customHeight="1" s="12">
+      <c r="I44" s="19" t="n"/>
+    </row>
+    <row r="45" ht="18" customHeight="1" s="12">
+      <c r="I45" s="19" t="n"/>
+    </row>
+    <row r="46" ht="18" customHeight="1" s="12">
+      <c r="I46" s="19" t="n"/>
+    </row>
+    <row r="47" ht="18" customHeight="1" s="12">
+      <c r="I47" s="19" t="n"/>
+    </row>
+    <row r="48" ht="18" customHeight="1" s="12">
+      <c r="I48" s="19" t="n"/>
+    </row>
+    <row r="49" ht="18" customHeight="1" s="12">
+      <c r="I49" s="19" t="n"/>
+    </row>
+    <row r="50" ht="18" customHeight="1" s="12">
+      <c r="I50" s="19" t="n"/>
+    </row>
+    <row r="51" ht="18" customHeight="1" s="12">
+      <c r="I51" s="19" t="n"/>
+    </row>
+    <row r="52" ht="18" customHeight="1" s="12">
+      <c r="I52" s="19" t="n"/>
+    </row>
+    <row r="53" ht="18" customHeight="1" s="12">
+      <c r="I53" s="19" t="n"/>
+    </row>
+    <row r="54" ht="18" customHeight="1" s="12">
+      <c r="I54" s="19" t="n"/>
+    </row>
+    <row r="55" ht="18" customHeight="1" s="12">
+      <c r="I55" s="19" t="n"/>
+    </row>
+    <row r="56" ht="18" customHeight="1" s="12">
+      <c r="I56" s="19" t="n"/>
+    </row>
+    <row r="57" ht="18" customHeight="1" s="12">
+      <c r="I57" s="19" t="n"/>
+    </row>
+    <row r="58" ht="18" customHeight="1" s="12">
+      <c r="I58" s="19" t="n"/>
+    </row>
+    <row r="59" ht="18" customHeight="1" s="12">
+      <c r="I59" s="19" t="n"/>
+    </row>
+    <row r="60" ht="18" customHeight="1" s="12">
+      <c r="I60" s="19" t="n"/>
+    </row>
+    <row r="61" ht="18" customHeight="1" s="12">
+      <c r="I61" s="19" t="n"/>
+    </row>
+    <row r="62" ht="18" customHeight="1" s="12">
+      <c r="I62" s="19" t="n"/>
+    </row>
+    <row r="63" ht="18" customHeight="1" s="12">
+      <c r="I63" s="19" t="n"/>
+    </row>
+    <row r="64" ht="18" customHeight="1" s="12">
+      <c r="I64" s="19" t="n"/>
+    </row>
+    <row r="65" ht="18" customHeight="1" s="12">
+      <c r="I65" s="19" t="n"/>
+    </row>
+    <row r="66" ht="18" customHeight="1" s="12">
+      <c r="I66" s="19" t="n"/>
+    </row>
+    <row r="67" ht="18" customHeight="1" s="12">
+      <c r="I67" s="19" t="n"/>
+    </row>
+    <row r="68" ht="18" customHeight="1" s="12">
+      <c r="I68" s="19" t="n"/>
+    </row>
+    <row r="69" ht="18" customHeight="1" s="12">
+      <c r="I69" s="19" t="n"/>
+    </row>
+    <row r="70" ht="18" customHeight="1" s="12">
+      <c r="I70" s="19" t="n"/>
+    </row>
+    <row r="71" ht="18" customHeight="1" s="12">
+      <c r="I71" s="19" t="n"/>
+    </row>
+    <row r="72" ht="18" customHeight="1" s="12">
+      <c r="I72" s="19" t="n"/>
+    </row>
+    <row r="73" ht="18" customHeight="1" s="12">
+      <c r="I73" s="19" t="n"/>
+    </row>
+    <row r="74" ht="18" customHeight="1" s="12">
+      <c r="I74" s="19" t="n"/>
+    </row>
+    <row r="75" ht="18" customHeight="1" s="12">
+      <c r="I75" s="19" t="n"/>
+    </row>
+    <row r="76" ht="18" customHeight="1" s="12">
+      <c r="I76" s="19" t="n"/>
+    </row>
+    <row r="77" ht="18" customHeight="1" s="12">
+      <c r="I77" s="19" t="n"/>
+    </row>
+    <row r="78" ht="18" customHeight="1" s="12">
+      <c r="I78" s="19" t="n"/>
+    </row>
+    <row r="79" ht="18" customHeight="1" s="12">
+      <c r="I79" s="19" t="n"/>
+    </row>
+    <row r="80" ht="18" customHeight="1" s="12">
+      <c r="I80" s="19" t="n"/>
+    </row>
+    <row r="81" ht="18" customHeight="1" s="12">
+      <c r="I81" s="19" t="n"/>
+    </row>
+    <row r="82" ht="18" customHeight="1" s="12">
+      <c r="I82" s="19" t="n"/>
+    </row>
+    <row r="83" ht="18" customHeight="1" s="12">
+      <c r="I83" s="19" t="n"/>
+    </row>
+    <row r="84" ht="18" customHeight="1" s="12">
+      <c r="I84" s="19" t="n"/>
+    </row>
+    <row r="85" ht="18" customHeight="1" s="12">
+      <c r="I85" s="19" t="n"/>
+    </row>
+    <row r="86" ht="18" customHeight="1" s="12">
+      <c r="I86" s="19" t="n"/>
+    </row>
+    <row r="87" ht="18" customHeight="1" s="12">
+      <c r="I87" s="19" t="n"/>
+    </row>
+    <row r="88" ht="18" customHeight="1" s="12">
+      <c r="I88" s="19" t="n"/>
+    </row>
+    <row r="89" ht="18" customHeight="1" s="12">
+      <c r="I89" s="19" t="n"/>
+    </row>
+    <row r="90" ht="18" customHeight="1" s="12">
+      <c r="I90" s="19" t="n"/>
+    </row>
+    <row r="91" ht="18" customHeight="1" s="12">
+      <c r="I91" s="19" t="n"/>
+    </row>
+    <row r="92" ht="18" customHeight="1" s="12">
+      <c r="I92" s="19" t="n"/>
+    </row>
+    <row r="93" ht="18" customHeight="1" s="12">
+      <c r="I93" s="19" t="n"/>
+    </row>
+    <row r="94" ht="18" customHeight="1" s="12">
+      <c r="I94" s="19" t="n"/>
+    </row>
+    <row r="95" ht="18" customHeight="1" s="12">
+      <c r="I95" s="19" t="n"/>
+    </row>
+    <row r="96" ht="18" customHeight="1" s="12">
+      <c r="I96" s="19" t="n"/>
+    </row>
+    <row r="97" ht="18" customHeight="1" s="12">
+      <c r="I97" s="19" t="n"/>
+    </row>
+    <row r="98" ht="18" customHeight="1" s="12">
+      <c r="I98" s="19" t="n"/>
+    </row>
+    <row r="99" ht="18" customHeight="1" s="12">
+      <c r="I99" s="19" t="n"/>
+    </row>
+    <row r="100" ht="18" customHeight="1" s="12">
+      <c r="I100" s="19" t="n"/>
+    </row>
+    <row r="101" ht="18" customHeight="1" s="12">
+      <c r="I101" s="19" t="n"/>
+    </row>
+    <row r="102" ht="18" customHeight="1" s="12">
+      <c r="I102" s="19" t="n"/>
+    </row>
+    <row r="103" ht="18" customHeight="1" s="12">
+      <c r="I103" s="19" t="n"/>
+    </row>
+    <row r="104" ht="18" customHeight="1" s="12">
+      <c r="I104" s="19" t="n"/>
+    </row>
+    <row r="105" ht="18" customHeight="1" s="12">
+      <c r="I105" s="19" t="n"/>
+    </row>
+    <row r="106" ht="18" customHeight="1" s="12">
+      <c r="I106" s="19" t="n"/>
+    </row>
+    <row r="107" ht="18" customHeight="1" s="12">
+      <c r="I107" s="19" t="n"/>
+    </row>
+    <row r="108" ht="18" customHeight="1" s="12">
+      <c r="I108" s="19" t="n"/>
+    </row>
+    <row r="109" ht="18" customHeight="1" s="12">
+      <c r="I109" s="19" t="n"/>
+    </row>
+    <row r="110" ht="18" customHeight="1" s="12">
+      <c r="I110" s="19" t="n"/>
+    </row>
+    <row r="111" ht="18" customHeight="1" s="12">
+      <c r="I111" s="19" t="n"/>
+    </row>
+    <row r="112" ht="18" customHeight="1" s="12">
+      <c r="I112" s="19" t="n"/>
+    </row>
+    <row r="113" ht="18" customHeight="1" s="12">
+      <c r="I113" s="19" t="n"/>
+    </row>
+    <row r="114" ht="18" customHeight="1" s="12">
+      <c r="I114" s="19" t="n"/>
+    </row>
+    <row r="115" ht="18" customHeight="1" s="12">
+      <c r="I115" s="19" t="n"/>
+    </row>
+    <row r="116" ht="18" customHeight="1" s="12">
+      <c r="I116" s="19" t="n"/>
+    </row>
+    <row r="117" ht="18" customHeight="1" s="12">
+      <c r="I117" s="19" t="n"/>
+    </row>
+    <row r="118" ht="18" customHeight="1" s="12">
+      <c r="I118" s="19" t="n"/>
+    </row>
+    <row r="119" ht="18" customHeight="1" s="12">
+      <c r="I119" s="19" t="n"/>
+    </row>
+    <row r="120" ht="18" customHeight="1" s="12">
+      <c r="I120" s="19" t="n"/>
+    </row>
+    <row r="121" ht="18" customHeight="1" s="12">
+      <c r="I121" s="19" t="n"/>
+    </row>
+    <row r="122" ht="18" customHeight="1" s="12">
+      <c r="I122" s="19" t="n"/>
+    </row>
+    <row r="123" ht="18" customHeight="1" s="12">
+      <c r="I123" s="19" t="n"/>
+    </row>
+    <row r="124" ht="18" customHeight="1" s="12">
+      <c r="I124" s="19" t="n"/>
+    </row>
+    <row r="125" ht="18" customHeight="1" s="12">
+      <c r="I125" s="19" t="n"/>
+    </row>
+    <row r="126" ht="18" customHeight="1" s="12">
+      <c r="I126" s="19" t="n"/>
+    </row>
+    <row r="127" ht="18" customHeight="1" s="12">
+      <c r="I127" s="19" t="n"/>
+    </row>
+    <row r="128" ht="18" customHeight="1" s="12">
+      <c r="I128" s="19" t="n"/>
+    </row>
+    <row r="129" ht="18" customHeight="1" s="12">
+      <c r="I129" s="19" t="n"/>
+    </row>
+    <row r="130" ht="18" customHeight="1" s="12">
+      <c r="I130" s="19" t="n"/>
+    </row>
+    <row r="131" ht="18" customHeight="1" s="12">
+      <c r="I131" s="19" t="n"/>
+    </row>
+    <row r="132" ht="18" customHeight="1" s="12">
+      <c r="I132" s="19" t="n"/>
+    </row>
+    <row r="133" ht="18" customHeight="1" s="12">
+      <c r="I133" s="19" t="n"/>
+    </row>
+    <row r="134" ht="18" customHeight="1" s="12">
+      <c r="I134" s="19" t="n"/>
+    </row>
+    <row r="135" ht="18" customHeight="1" s="12">
+      <c r="I135" s="19" t="n"/>
+    </row>
+    <row r="136" ht="18" customHeight="1" s="12">
+      <c r="I136" s="19" t="n"/>
+    </row>
+    <row r="137" ht="18" customHeight="1" s="12">
+      <c r="I137" s="19" t="n"/>
+    </row>
+    <row r="138" ht="18" customHeight="1" s="12">
+      <c r="I138" s="19" t="n"/>
+    </row>
+    <row r="139" ht="18" customHeight="1" s="12">
+      <c r="I139" s="19" t="n"/>
+    </row>
+    <row r="140" ht="18" customHeight="1" s="12">
+      <c r="I140" s="19" t="n"/>
+    </row>
+    <row r="141" ht="18" customHeight="1" s="12">
+      <c r="I141" s="19" t="n"/>
+    </row>
+    <row r="142" ht="18" customHeight="1" s="12">
+      <c r="I142" s="19" t="n"/>
+    </row>
+    <row r="143" ht="18" customHeight="1" s="12">
+      <c r="I143" s="19" t="n"/>
+    </row>
+    <row r="144" ht="18" customHeight="1" s="12">
+      <c r="I144" s="19" t="n"/>
+    </row>
+    <row r="145" ht="18" customHeight="1" s="12">
+      <c r="I145" s="19" t="n"/>
+    </row>
+    <row r="146" ht="18" customHeight="1" s="12">
+      <c r="I146" s="19" t="n"/>
+    </row>
+    <row r="147" ht="18" customHeight="1" s="12">
+      <c r="I147" s="19" t="n"/>
+    </row>
+    <row r="148" ht="18" customHeight="1" s="12">
+      <c r="I148" s="19" t="n"/>
+    </row>
+    <row r="149" ht="18" customHeight="1" s="12">
+      <c r="I149" s="19" t="n"/>
+    </row>
+    <row r="150" ht="18" customHeight="1" s="12">
+      <c r="I150" s="19" t="n"/>
+    </row>
+    <row r="151" ht="18" customHeight="1" s="12">
+      <c r="I151" s="19" t="n"/>
+    </row>
+    <row r="152" ht="18" customHeight="1" s="12">
+      <c r="I152" s="19" t="n"/>
+    </row>
+    <row r="153" ht="18" customHeight="1" s="12">
+      <c r="I153" s="19" t="n"/>
+    </row>
+    <row r="154" ht="18" customHeight="1" s="12">
+      <c r="I154" s="19" t="n"/>
+    </row>
+    <row r="155" ht="18" customHeight="1" s="12">
+      <c r="I155" s="19" t="n"/>
+    </row>
+    <row r="156" ht="18" customHeight="1" s="12">
+      <c r="I156" s="19" t="n"/>
+    </row>
+    <row r="157" ht="18" customHeight="1" s="12">
+      <c r="I157" s="19" t="n"/>
+    </row>
+    <row r="158" ht="18" customHeight="1" s="12">
+      <c r="I158" s="19" t="n"/>
+    </row>
+    <row r="159" ht="18" customHeight="1" s="12">
+      <c r="I159" s="19" t="n"/>
+    </row>
+    <row r="160" ht="18" customHeight="1" s="12">
+      <c r="I160" s="19" t="n"/>
+    </row>
+    <row r="161" ht="18" customHeight="1" s="12">
+      <c r="I161" s="19" t="n"/>
+    </row>
+    <row r="162" ht="18" customHeight="1" s="12">
+      <c r="I162" s="19" t="n"/>
+    </row>
+    <row r="163" ht="18" customHeight="1" s="12">
+      <c r="I163" s="19" t="n"/>
+    </row>
+    <row r="164" ht="18" customHeight="1" s="12">
+      <c r="I164" s="19" t="n"/>
+    </row>
+    <row r="165" ht="18" customHeight="1" s="12">
+      <c r="I165" s="19" t="n"/>
+    </row>
+    <row r="166" ht="18" customHeight="1" s="12">
+      <c r="I166" s="19" t="n"/>
+    </row>
+    <row r="167" ht="18" customHeight="1" s="12">
+      <c r="I167" s="19" t="n"/>
+    </row>
+    <row r="168" ht="18" customHeight="1" s="12">
+      <c r="I168" s="19" t="n"/>
+    </row>
+    <row r="169" ht="18" customHeight="1" s="12">
+      <c r="I169" s="19" t="n"/>
+    </row>
+    <row r="170" ht="18" customHeight="1" s="12">
+      <c r="I170" s="19" t="n"/>
+    </row>
+    <row r="171" ht="18" customHeight="1" s="12">
+      <c r="I171" s="19" t="n"/>
+    </row>
+    <row r="172" ht="18" customHeight="1" s="12">
+      <c r="I172" s="19" t="n"/>
+    </row>
+    <row r="173" ht="18" customHeight="1" s="12">
+      <c r="I173" s="19" t="n"/>
+    </row>
+    <row r="174" ht="18" customHeight="1" s="12">
+      <c r="I174" s="19" t="n"/>
+    </row>
+    <row r="175" ht="18" customHeight="1" s="12">
+      <c r="I175" s="19" t="n"/>
+    </row>
+    <row r="176" ht="18" customHeight="1" s="12">
+      <c r="I176" s="19" t="n"/>
+    </row>
+    <row r="177" ht="18" customHeight="1" s="12">
+      <c r="I177" s="19" t="n"/>
+    </row>
+    <row r="178" ht="18" customHeight="1" s="12">
+      <c r="I178" s="19" t="n"/>
+    </row>
+    <row r="179" ht="18" customHeight="1" s="12">
+      <c r="I179" s="19" t="n"/>
+    </row>
+    <row r="180" ht="18" customHeight="1" s="12">
+      <c r="I180" s="19" t="n"/>
+    </row>
+    <row r="181" ht="18" customHeight="1" s="12">
+      <c r="I181" s="19" t="n"/>
+    </row>
+    <row r="182" ht="18" customHeight="1" s="12">
+      <c r="I182" s="19" t="n"/>
+    </row>
+    <row r="183" ht="18" customHeight="1" s="12">
+      <c r="I183" s="19" t="n"/>
+    </row>
+    <row r="184" ht="18" customHeight="1" s="12">
+      <c r="I184" s="19" t="n"/>
+    </row>
+    <row r="185" ht="18" customHeight="1" s="12">
+      <c r="I185" s="19" t="n"/>
+    </row>
+    <row r="186" ht="18" customHeight="1" s="12">
+      <c r="I186" s="19" t="n"/>
+    </row>
+    <row r="187" ht="18" customHeight="1" s="12">
+      <c r="I187" s="19" t="n"/>
+    </row>
+    <row r="188" ht="18" customHeight="1" s="12">
+      <c r="I188" s="19" t="n"/>
+    </row>
+    <row r="189" ht="18" customHeight="1" s="12">
+      <c r="I189" s="19" t="n"/>
+    </row>
+    <row r="190" ht="18" customHeight="1" s="12">
+      <c r="I190" s="19" t="n"/>
+    </row>
+    <row r="191" ht="18" customHeight="1" s="12">
+      <c r="I191" s="19" t="n"/>
+    </row>
+    <row r="192" ht="18" customHeight="1" s="12">
+      <c r="I192" s="19" t="n"/>
+    </row>
+    <row r="193" ht="18" customHeight="1" s="12">
+      <c r="I193" s="19" t="n"/>
+    </row>
+    <row r="194" ht="18" customHeight="1" s="12">
+      <c r="I194" s="19" t="n"/>
+    </row>
+    <row r="195" ht="18" customHeight="1" s="12">
+      <c r="I195" s="19" t="n"/>
+    </row>
+    <row r="196" ht="18" customHeight="1" s="12">
+      <c r="I196" s="19" t="n"/>
+    </row>
+    <row r="197" ht="18" customHeight="1" s="12">
+      <c r="I197" s="19" t="n"/>
+    </row>
+    <row r="198" ht="18" customHeight="1" s="12">
+      <c r="I198" s="19" t="n"/>
+    </row>
+    <row r="199" ht="18" customHeight="1" s="12">
+      <c r="I199" s="19" t="n"/>
+    </row>
+    <row r="200" ht="18" customHeight="1" s="12">
+      <c r="I200" s="19" t="n"/>
+    </row>
+    <row r="201" ht="18" customHeight="1" s="12">
+      <c r="I201" s="19" t="n"/>
+    </row>
+    <row r="202" ht="18" customHeight="1" s="12">
+      <c r="I202" s="19" t="n"/>
+    </row>
+    <row r="203" ht="18" customHeight="1" s="12">
+      <c r="I203" s="19" t="n"/>
+    </row>
+    <row r="204" ht="18" customHeight="1" s="12">
+      <c r="I204" s="19" t="n"/>
+    </row>
+    <row r="205" ht="18" customHeight="1" s="12">
+      <c r="I205" s="19" t="n"/>
+    </row>
+    <row r="206" ht="18" customHeight="1" s="12">
+      <c r="I206" s="19" t="n"/>
+    </row>
+    <row r="207" ht="18" customHeight="1" s="12">
+      <c r="I207" s="19" t="n"/>
+    </row>
+    <row r="208" ht="18" customHeight="1" s="12">
+      <c r="I208" s="19" t="n"/>
+    </row>
+    <row r="209" ht="18" customHeight="1" s="12">
+      <c r="I209" s="19" t="n"/>
+    </row>
+    <row r="210" ht="18" customHeight="1" s="12">
+      <c r="I210" s="19" t="n"/>
+    </row>
+    <row r="211" ht="18" customHeight="1" s="12">
+      <c r="I211" s="19" t="n"/>
+    </row>
+    <row r="212" ht="18" customHeight="1" s="12">
+      <c r="I212" s="19" t="n"/>
+    </row>
+    <row r="213" ht="18" customHeight="1" s="12">
+      <c r="I213" s="19" t="n"/>
+    </row>
+    <row r="214" ht="18" customHeight="1" s="12">
+      <c r="I214" s="19" t="n"/>
+    </row>
+    <row r="215" ht="18" customHeight="1" s="12">
+      <c r="I215" s="19" t="n"/>
+    </row>
+    <row r="216" ht="18" customHeight="1" s="12">
+      <c r="I216" s="19" t="n"/>
+    </row>
+    <row r="217" ht="18" customHeight="1" s="12">
+      <c r="I217" s="19" t="n"/>
+    </row>
+    <row r="218" ht="18" customHeight="1" s="12">
+      <c r="I218" s="19" t="n"/>
+    </row>
+    <row r="219" ht="18" customHeight="1" s="12">
+      <c r="I219" s="19" t="n"/>
+    </row>
+    <row r="220" ht="18" customHeight="1" s="12">
+      <c r="I220" s="19" t="n"/>
+    </row>
+    <row r="221" ht="18" customHeight="1" s="12">
+      <c r="I221" s="19" t="n"/>
+    </row>
+    <row r="222" ht="18" customHeight="1" s="12">
+      <c r="I222" s="19" t="n"/>
+    </row>
+    <row r="223" ht="18" customHeight="1" s="12">
+      <c r="I223" s="19" t="n"/>
+    </row>
+    <row r="224" ht="18" customHeight="1" s="12">
+      <c r="I224" s="19" t="n"/>
+    </row>
+    <row r="225" ht="18" customHeight="1" s="12">
+      <c r="I225" s="19" t="n"/>
+    </row>
+    <row r="226" ht="18" customHeight="1" s="12">
+      <c r="I226" s="19" t="n"/>
+    </row>
+    <row r="227" ht="18" customHeight="1" s="12">
+      <c r="I227" s="19" t="n"/>
+    </row>
+    <row r="228" ht="18" customHeight="1" s="12">
+      <c r="I228" s="19" t="n"/>
+    </row>
+    <row r="229" ht="18" customHeight="1" s="12">
+      <c r="I229" s="19" t="n"/>
+    </row>
+    <row r="230" ht="18" customHeight="1" s="12">
+      <c r="I230" s="19" t="n"/>
+    </row>
+    <row r="231" ht="18" customHeight="1" s="12">
+      <c r="I231" s="19" t="n"/>
+    </row>
+    <row r="232" ht="18" customHeight="1" s="12">
+      <c r="I232" s="19" t="n"/>
+    </row>
+    <row r="233" ht="18" customHeight="1" s="12">
+      <c r="I233" s="19" t="n"/>
+    </row>
+    <row r="234" ht="18" customHeight="1" s="12">
+      <c r="I234" s="19" t="n"/>
+    </row>
+    <row r="235" ht="18" customHeight="1" s="12">
+      <c r="I235" s="19" t="n"/>
+    </row>
+    <row r="236" ht="18" customHeight="1" s="12">
+      <c r="I236" s="19" t="n"/>
+    </row>
+    <row r="237" ht="18" customHeight="1" s="12">
+      <c r="I237" s="19" t="n"/>
+    </row>
+    <row r="238" ht="18" customHeight="1" s="12">
+      <c r="I238" s="19" t="n"/>
+    </row>
+    <row r="239" ht="18" customHeight="1" s="12">
+      <c r="I239" s="19" t="n"/>
+    </row>
+    <row r="240" ht="18" customHeight="1" s="12">
+      <c r="I240" s="19" t="n"/>
+    </row>
+    <row r="241" ht="18" customHeight="1" s="12">
+      <c r="I241" s="19" t="n"/>
+    </row>
+    <row r="242" ht="18" customHeight="1" s="12">
+      <c r="I242" s="19" t="n"/>
+    </row>
+    <row r="243" ht="18" customHeight="1" s="12">
+      <c r="I243" s="19" t="n"/>
+    </row>
+    <row r="244" ht="18" customHeight="1" s="12">
+      <c r="I244" s="19" t="n"/>
+    </row>
+    <row r="245" ht="18" customHeight="1" s="12">
+      <c r="I245" s="19" t="n"/>
+    </row>
+    <row r="246" ht="18" customHeight="1" s="12">
+      <c r="I246" s="19" t="n"/>
+    </row>
+    <row r="247" ht="18" customHeight="1" s="12">
+      <c r="I247" s="19" t="n"/>
+    </row>
+    <row r="248" ht="18" customHeight="1" s="12">
+      <c r="I248" s="19" t="n"/>
+    </row>
+    <row r="249" ht="18" customHeight="1" s="12">
+      <c r="I249" s="19" t="n"/>
+    </row>
+    <row r="250" ht="18" customHeight="1" s="12">
+      <c r="I250" s="19" t="n"/>
+    </row>
+    <row r="251" ht="18" customHeight="1" s="12">
+      <c r="I251" s="19" t="n"/>
+    </row>
+    <row r="252" ht="18" customHeight="1" s="12">
+      <c r="I252" s="19" t="n"/>
+    </row>
+    <row r="253" ht="18" customHeight="1" s="12">
+      <c r="I253" s="19" t="n"/>
+    </row>
+    <row r="254" ht="18" customHeight="1" s="12">
+      <c r="I254" s="19" t="n"/>
+    </row>
+    <row r="255" ht="18" customHeight="1" s="12">
+      <c r="I255" s="19" t="n"/>
+    </row>
+    <row r="256" ht="18" customHeight="1" s="12">
+      <c r="I256" s="19" t="n"/>
+    </row>
+    <row r="257" ht="18" customHeight="1" s="12">
+      <c r="I257" s="19" t="n"/>
+    </row>
+    <row r="258" ht="18" customHeight="1" s="12">
+      <c r="I258" s="19" t="n"/>
+    </row>
+    <row r="259" ht="18" customHeight="1" s="12">
+      <c r="I259" s="19" t="n"/>
+    </row>
+    <row r="260" ht="18" customHeight="1" s="12">
+      <c r="I260" s="19" t="n"/>
+    </row>
+    <row r="261" ht="18" customHeight="1" s="12">
+      <c r="I261" s="19" t="n"/>
+    </row>
+    <row r="262" ht="18" customHeight="1" s="12">
+      <c r="I262" s="19" t="n"/>
+    </row>
+    <row r="263" ht="18" customHeight="1" s="12">
+      <c r="I263" s="19" t="n"/>
+    </row>
+    <row r="264" ht="18" customHeight="1" s="12">
+      <c r="I264" s="19" t="n"/>
+    </row>
+    <row r="265" ht="18" customHeight="1" s="12">
+      <c r="I265" s="19" t="n"/>
+    </row>
+    <row r="266" ht="18" customHeight="1" s="12">
+      <c r="I266" s="19" t="n"/>
+    </row>
+    <row r="267" ht="18" customHeight="1" s="12">
+      <c r="I267" s="19" t="n"/>
+    </row>
+    <row r="268" ht="18" customHeight="1" s="12">
+      <c r="I268" s="19" t="n"/>
+    </row>
+    <row r="269" ht="18" customHeight="1" s="12">
+      <c r="I269" s="19" t="n"/>
+    </row>
+    <row r="270" ht="18" customHeight="1" s="12">
+      <c r="I270" s="19" t="n"/>
+    </row>
+    <row r="271" ht="18" customHeight="1" s="12">
+      <c r="I271" s="19" t="n"/>
+    </row>
+    <row r="272" ht="18" customHeight="1" s="12">
+      <c r="I272" s="19" t="n"/>
+    </row>
+    <row r="273" ht="18" customHeight="1" s="12">
+      <c r="I273" s="19" t="n"/>
+    </row>
+    <row r="274" ht="18" customHeight="1" s="12">
+      <c r="I274" s="19" t="n"/>
+    </row>
+    <row r="275" ht="18" customHeight="1" s="12">
+      <c r="I275" s="19" t="n"/>
+    </row>
+    <row r="276" ht="18" customHeight="1" s="12">
+      <c r="I276" s="19" t="n"/>
+    </row>
+    <row r="277" ht="18" customHeight="1" s="12">
+      <c r="I277" s="19" t="n"/>
+    </row>
+    <row r="278" ht="18" customHeight="1" s="12">
+      <c r="I278" s="19" t="n"/>
+    </row>
+    <row r="279" ht="18" customHeight="1" s="12">
+      <c r="I279" s="19" t="n"/>
+    </row>
+    <row r="280" ht="18" customHeight="1" s="12">
+      <c r="I280" s="19" t="n"/>
+    </row>
+    <row r="281" ht="18" customHeight="1" s="12">
+      <c r="I281" s="19" t="n"/>
+    </row>
+    <row r="282" ht="18" customHeight="1" s="12">
+      <c r="I282" s="19" t="n"/>
+    </row>
+    <row r="283" ht="18" customHeight="1" s="12">
+      <c r="I283" s="19" t="n"/>
+    </row>
+    <row r="284" ht="18" customHeight="1" s="12">
+      <c r="I284" s="19" t="n"/>
+    </row>
+    <row r="285" ht="18" customHeight="1" s="12">
+      <c r="I285" s="19" t="n"/>
+    </row>
+    <row r="286" ht="18" customHeight="1" s="12">
+      <c r="I286" s="19" t="n"/>
+    </row>
+    <row r="287" ht="18" customHeight="1" s="12">
+      <c r="I287" s="19" t="n"/>
+    </row>
+    <row r="288" ht="18" customHeight="1" s="12">
+      <c r="I288" s="19" t="n"/>
+    </row>
+    <row r="289" ht="18" customHeight="1" s="12">
+      <c r="I289" s="19" t="n"/>
+    </row>
+    <row r="290" ht="18" customHeight="1" s="12">
+      <c r="I290" s="19" t="n"/>
+    </row>
+    <row r="291" ht="18" customHeight="1" s="12">
+      <c r="I291" s="19" t="n"/>
+    </row>
+    <row r="292" ht="18" customHeight="1" s="12">
+      <c r="I292" s="19" t="n"/>
+    </row>
+    <row r="293" ht="18" customHeight="1" s="12">
+      <c r="I293" s="19" t="n"/>
+    </row>
+    <row r="294" ht="18" customHeight="1" s="12">
+      <c r="I294" s="19" t="n"/>
+    </row>
+    <row r="295" ht="18" customHeight="1" s="12">
+      <c r="I295" s="19" t="n"/>
+    </row>
+    <row r="296" ht="18" customHeight="1" s="12">
+      <c r="I296" s="19" t="n"/>
+    </row>
+    <row r="297" ht="18" customHeight="1" s="12">
+      <c r="I297" s="19" t="n"/>
+    </row>
+    <row r="298" ht="18" customHeight="1" s="12">
+      <c r="I298" s="19" t="n"/>
+    </row>
+    <row r="299" ht="18" customHeight="1" s="12">
+      <c r="I299" s="19" t="n"/>
+    </row>
+    <row r="300" ht="18" customHeight="1" s="12">
+      <c r="I300" s="19" t="n"/>
+    </row>
+    <row r="301" ht="18" customHeight="1" s="12">
+      <c r="I301" s="19" t="n"/>
+    </row>
+    <row r="302" ht="18" customHeight="1" s="12">
+      <c r="I302" s="19" t="n"/>
+    </row>
+    <row r="303" ht="18" customHeight="1" s="12">
+      <c r="I303" s="19" t="n"/>
+    </row>
+    <row r="304" ht="18" customHeight="1" s="12">
+      <c r="I304" s="19" t="n"/>
+    </row>
+    <row r="305" ht="18" customHeight="1" s="12">
+      <c r="I305" s="19" t="n"/>
+    </row>
+    <row r="306" ht="18" customHeight="1" s="12">
+      <c r="I306" s="19" t="n"/>
+    </row>
+    <row r="307" ht="18" customHeight="1" s="12">
+      <c r="I307" s="19" t="n"/>
+    </row>
+    <row r="308" ht="18" customHeight="1" s="12">
+      <c r="I308" s="19" t="n"/>
+    </row>
+    <row r="309" ht="18" customHeight="1" s="12">
+      <c r="I309" s="19" t="n"/>
+    </row>
+    <row r="310" ht="18" customHeight="1" s="12">
+      <c r="I310" s="19" t="n"/>
+    </row>
+    <row r="311" ht="18" customHeight="1" s="12">
+      <c r="I311" s="19" t="n"/>
+    </row>
+    <row r="312" ht="18" customHeight="1" s="12">
+      <c r="I312" s="19" t="n"/>
+    </row>
+    <row r="313" ht="18" customHeight="1" s="12">
+      <c r="I313" s="19" t="n"/>
+    </row>
+    <row r="314" ht="18" customHeight="1" s="12">
+      <c r="I314" s="19" t="n"/>
+    </row>
+    <row r="315" ht="18" customHeight="1" s="12">
+      <c r="I315" s="19" t="n"/>
+    </row>
+    <row r="316" ht="18" customHeight="1" s="12">
+      <c r="I316" s="19" t="n"/>
+    </row>
+    <row r="317" ht="18" customHeight="1" s="12">
+      <c r="I317" s="19" t="n"/>
+    </row>
+    <row r="318" ht="18" customHeight="1" s="12">
+      <c r="I318" s="19" t="n"/>
+    </row>
+    <row r="319" ht="18" customHeight="1" s="12">
+      <c r="I319" s="19" t="n"/>
+    </row>
+    <row r="320" ht="18" customHeight="1" s="12">
+      <c r="I320" s="19" t="n"/>
+    </row>
+    <row r="321" ht="18" customHeight="1" s="12">
+      <c r="I321" s="19" t="n"/>
+    </row>
+    <row r="322" ht="18" customHeight="1" s="12">
+      <c r="I322" s="19" t="n"/>
+    </row>
+    <row r="323" ht="18" customHeight="1" s="12">
+      <c r="I323" s="19" t="n"/>
+    </row>
+    <row r="324" ht="18" customHeight="1" s="12">
+      <c r="I324" s="19" t="n"/>
+    </row>
+    <row r="325" ht="18" customHeight="1" s="12">
+      <c r="I325" s="19" t="n"/>
+    </row>
+    <row r="326" ht="18" customHeight="1" s="12">
+      <c r="I326" s="19" t="n"/>
+    </row>
+    <row r="327" ht="18" customHeight="1" s="12">
+      <c r="I327" s="19" t="n"/>
+    </row>
+    <row r="328" ht="18" customHeight="1" s="12">
+      <c r="I328" s="19" t="n"/>
+    </row>
+    <row r="329" ht="18" customHeight="1" s="12">
+      <c r="I329" s="19" t="n"/>
+    </row>
+    <row r="330" ht="18" customHeight="1" s="12">
+      <c r="I330" s="19" t="n"/>
+    </row>
+    <row r="331" ht="18" customHeight="1" s="12">
+      <c r="I331" s="19" t="n"/>
+    </row>
+    <row r="332" ht="18" customHeight="1" s="12">
+      <c r="I332" s="19" t="n"/>
+    </row>
+    <row r="333" ht="18" customHeight="1" s="12">
+      <c r="I333" s="19" t="n"/>
+    </row>
+    <row r="334" ht="18" customHeight="1" s="12">
+      <c r="I334" s="19" t="n"/>
+    </row>
+    <row r="335" ht="18" customHeight="1" s="12">
+      <c r="I335" s="19" t="n"/>
+    </row>
+    <row r="336" ht="18" customHeight="1" s="12">
+      <c r="I336" s="19" t="n"/>
+    </row>
+    <row r="337" ht="18" customHeight="1" s="12">
+      <c r="I337" s="19" t="n"/>
+    </row>
+    <row r="338" ht="18" customHeight="1" s="12">
+      <c r="I338" s="19" t="n"/>
+    </row>
+    <row r="339" ht="18" customHeight="1" s="12">
+      <c r="I339" s="19" t="n"/>
+    </row>
+    <row r="340" ht="18" customHeight="1" s="12">
+      <c r="I340" s="19" t="n"/>
+    </row>
+    <row r="341" ht="18" customHeight="1" s="12">
+      <c r="I341" s="19" t="n"/>
+    </row>
+    <row r="342" ht="18" customHeight="1" s="12">
+      <c r="I342" s="19" t="n"/>
+    </row>
+    <row r="343" ht="18" customHeight="1" s="12">
+      <c r="I343" s="19" t="n"/>
+    </row>
+    <row r="344" ht="18" customHeight="1" s="12">
+      <c r="I344" s="19" t="n"/>
+    </row>
+    <row r="345" ht="18" customHeight="1" s="12">
+      <c r="I345" s="19" t="n"/>
+    </row>
+    <row r="346" ht="18" customHeight="1" s="12">
+      <c r="I346" s="19" t="n"/>
+    </row>
+    <row r="347" ht="18" customHeight="1" s="12">
+      <c r="I347" s="19" t="n"/>
+    </row>
+    <row r="348" ht="18" customHeight="1" s="12">
+      <c r="I348" s="19" t="n"/>
+    </row>
+    <row r="349" ht="18" customHeight="1" s="12">
+      <c r="I349" s="19" t="n"/>
+    </row>
+    <row r="350" ht="18" customHeight="1" s="12">
+      <c r="I350" s="19" t="n"/>
+    </row>
+    <row r="351" ht="18" customHeight="1" s="12">
+      <c r="I351" s="19" t="n"/>
+    </row>
+    <row r="352" ht="18" customHeight="1" s="12">
+      <c r="I352" s="19" t="n"/>
+    </row>
+    <row r="353" ht="18" customHeight="1" s="12">
+      <c r="I353" s="19" t="n"/>
+    </row>
+    <row r="354" ht="18" customHeight="1" s="12">
+      <c r="I354" s="19" t="n"/>
+    </row>
+    <row r="355" ht="18" customHeight="1" s="12">
+      <c r="I355" s="19" t="n"/>
+    </row>
+    <row r="356" ht="18" customHeight="1" s="12">
+      <c r="I356" s="19" t="n"/>
+    </row>
+    <row r="357" ht="18" customHeight="1" s="12">
+      <c r="I357" s="19" t="n"/>
+    </row>
+    <row r="358" ht="18" customHeight="1" s="12">
+      <c r="I358" s="19" t="n"/>
+    </row>
+    <row r="359" ht="18" customHeight="1" s="12">
+      <c r="I359" s="19" t="n"/>
+    </row>
+    <row r="360" ht="18" customHeight="1" s="12">
+      <c r="I360" s="19" t="n"/>
+    </row>
+    <row r="361" ht="18" customHeight="1" s="12">
+      <c r="I361" s="19" t="n"/>
+    </row>
+    <row r="362" ht="18" customHeight="1" s="12">
+      <c r="I362" s="19" t="n"/>
+    </row>
+    <row r="363" ht="18" customHeight="1" s="12">
+      <c r="I363" s="19" t="n"/>
+    </row>
+    <row r="364" ht="18" customHeight="1" s="12">
+      <c r="I364" s="19" t="n"/>
+    </row>
+    <row r="365" ht="18" customHeight="1" s="12">
+      <c r="I365" s="19" t="n"/>
+    </row>
+    <row r="366" ht="18" customHeight="1" s="12">
+      <c r="I366" s="19" t="n"/>
+    </row>
+    <row r="367" ht="18" customHeight="1" s="12">
+      <c r="I367" s="19" t="n"/>
+    </row>
+    <row r="368" ht="18" customHeight="1" s="12">
+      <c r="I368" s="19" t="n"/>
+    </row>
+    <row r="369" ht="18" customHeight="1" s="12">
+      <c r="I369" s="19" t="n"/>
+    </row>
+    <row r="370" ht="18" customHeight="1" s="12">
+      <c r="I370" s="19" t="n"/>
+    </row>
+    <row r="371" ht="18" customHeight="1" s="12">
+      <c r="I371" s="19" t="n"/>
+    </row>
+    <row r="372" ht="18" customHeight="1" s="12">
+      <c r="I372" s="19" t="n"/>
+    </row>
+    <row r="373" ht="18" customHeight="1" s="12">
+      <c r="I373" s="19" t="n"/>
+    </row>
+    <row r="374" ht="18" customHeight="1" s="12">
+      <c r="I374" s="19" t="n"/>
+    </row>
+    <row r="375" ht="18" customHeight="1" s="12">
+      <c r="I375" s="19" t="n"/>
+    </row>
+    <row r="376" ht="18" customHeight="1" s="12">
+      <c r="I376" s="19" t="n"/>
+    </row>
+    <row r="377" ht="18" customHeight="1" s="12">
+      <c r="I377" s="19" t="n"/>
+    </row>
+    <row r="378" ht="18" customHeight="1" s="12">
+      <c r="I378" s="19" t="n"/>
+    </row>
+    <row r="379" ht="18" customHeight="1" s="12">
+      <c r="I379" s="19" t="n"/>
+    </row>
+    <row r="380" ht="18" customHeight="1" s="12">
+      <c r="I380" s="19" t="n"/>
+    </row>
+    <row r="381" ht="18" customHeight="1" s="12">
+      <c r="I381" s="19" t="n"/>
+    </row>
+    <row r="382" ht="18" customHeight="1" s="12">
+      <c r="I382" s="19" t="n"/>
+    </row>
+    <row r="383" ht="18" customHeight="1" s="12">
+      <c r="I383" s="19" t="n"/>
+    </row>
+    <row r="384" ht="18" customHeight="1" s="12">
+      <c r="I384" s="19" t="n"/>
+    </row>
+    <row r="385" ht="18" customHeight="1" s="12">
+      <c r="I385" s="19" t="n"/>
+    </row>
+    <row r="386" ht="18" customHeight="1" s="12">
+      <c r="I386" s="19" t="n"/>
+    </row>
+    <row r="387" ht="18" customHeight="1" s="12">
+      <c r="I387" s="19" t="n"/>
+    </row>
+    <row r="388" ht="18" customHeight="1" s="12">
+      <c r="I388" s="19" t="n"/>
+    </row>
+    <row r="389" ht="18" customHeight="1" s="12">
+      <c r="I389" s="19" t="n"/>
+    </row>
+    <row r="390" ht="18" customHeight="1" s="12">
+      <c r="I390" s="19" t="n"/>
+    </row>
+    <row r="391" ht="18" customHeight="1" s="12">
+      <c r="I391" s="19" t="n"/>
+    </row>
+    <row r="392" ht="18" customHeight="1" s="12">
+      <c r="I392" s="19" t="n"/>
+    </row>
+    <row r="393" ht="18" customHeight="1" s="12">
+      <c r="I393" s="19" t="n"/>
+    </row>
+    <row r="394" ht="18" customHeight="1" s="12">
+      <c r="I394" s="19" t="n"/>
+    </row>
+    <row r="395" ht="18" customHeight="1" s="12">
+      <c r="I395" s="19" t="n"/>
+    </row>
+    <row r="396" ht="18" customHeight="1" s="12">
+      <c r="I396" s="19" t="n"/>
+    </row>
+    <row r="397" ht="18" customHeight="1" s="12">
+      <c r="I397" s="19" t="n"/>
+    </row>
+    <row r="398" ht="18" customHeight="1" s="12">
+      <c r="I398" s="19" t="n"/>
+    </row>
+    <row r="399" ht="18" customHeight="1" s="12">
+      <c r="I399" s="19" t="n"/>
+    </row>
+    <row r="400" ht="18" customHeight="1" s="12">
+      <c r="I400" s="19" t="n"/>
+    </row>
+    <row r="401" ht="18" customHeight="1" s="12">
+      <c r="I401" s="19" t="n"/>
+    </row>
+    <row r="402" ht="18" customHeight="1" s="12">
+      <c r="I402" s="19" t="n"/>
+    </row>
+    <row r="403" ht="18" customHeight="1" s="12">
+      <c r="I403" s="19" t="n"/>
+    </row>
+    <row r="404" ht="18" customHeight="1" s="12">
+      <c r="I404" s="19" t="n"/>
+    </row>
+    <row r="405" ht="18" customHeight="1" s="12">
+      <c r="I405" s="19" t="n"/>
+    </row>
+    <row r="406" ht="18" customHeight="1" s="12">
+      <c r="I406" s="19" t="n"/>
+    </row>
+    <row r="407" ht="18" customHeight="1" s="12">
+      <c r="I407" s="19" t="n"/>
+    </row>
+    <row r="408" ht="18" customHeight="1" s="12">
+      <c r="I408" s="19" t="n"/>
+    </row>
+    <row r="409" ht="18" customHeight="1" s="12">
+      <c r="I409" s="19" t="n"/>
+    </row>
+    <row r="410" ht="18" customHeight="1" s="12">
+      <c r="I410" s="19" t="n"/>
+    </row>
+    <row r="411" ht="18" customHeight="1" s="12">
+      <c r="I411" s="19" t="n"/>
+    </row>
+    <row r="412" ht="18" customHeight="1" s="12">
+      <c r="I412" s="19" t="n"/>
+    </row>
+    <row r="413" ht="18" customHeight="1" s="12">
+      <c r="I413" s="19" t="n"/>
+    </row>
+    <row r="414" ht="18" customHeight="1" s="12">
+      <c r="I414" s="19" t="n"/>
+    </row>
+    <row r="415" ht="18" customHeight="1" s="12">
+      <c r="I415" s="19" t="n"/>
+    </row>
+    <row r="416" ht="18" customHeight="1" s="12">
+      <c r="I416" s="19" t="n"/>
+    </row>
+    <row r="417" ht="18" customHeight="1" s="12">
+      <c r="I417" s="19" t="n"/>
+    </row>
+    <row r="418" ht="18" customHeight="1" s="12">
+      <c r="I418" s="19" t="n"/>
+    </row>
+    <row r="419" ht="18" customHeight="1" s="12">
+      <c r="I419" s="19" t="n"/>
+    </row>
+    <row r="420" ht="18" customHeight="1" s="12">
+      <c r="I420" s="19" t="n"/>
+    </row>
+    <row r="421" ht="18" customHeight="1" s="12">
+      <c r="I421" s="19" t="n"/>
+    </row>
+    <row r="422" ht="18" customHeight="1" s="12">
+      <c r="I422" s="19" t="n"/>
+    </row>
+    <row r="423" ht="18" customHeight="1" s="12">
+      <c r="I423" s="19" t="n"/>
+    </row>
+    <row r="424" ht="18" customHeight="1" s="12">
+      <c r="I424" s="19" t="n"/>
+    </row>
+    <row r="425" ht="18" customHeight="1" s="12">
+      <c r="I425" s="19" t="n"/>
+    </row>
+    <row r="426" ht="18" customHeight="1" s="12">
+      <c r="I426" s="19" t="n"/>
+    </row>
+    <row r="427" ht="18" customHeight="1" s="12">
+      <c r="I427" s="19" t="n"/>
+    </row>
+    <row r="428" ht="18" customHeight="1" s="12">
+      <c r="I428" s="19" t="n"/>
+    </row>
+    <row r="429" ht="18" customHeight="1" s="12">
+      <c r="I429" s="19" t="n"/>
+    </row>
+    <row r="430" ht="18" customHeight="1" s="12">
+      <c r="I430" s="19" t="n"/>
+    </row>
+    <row r="431" ht="18" customHeight="1" s="12">
+      <c r="I431" s="19" t="n"/>
+    </row>
+    <row r="432" ht="18" customHeight="1" s="12">
+      <c r="I432" s="19" t="n"/>
+    </row>
+    <row r="433" ht="18" customHeight="1" s="12">
+      <c r="I433" s="19" t="n"/>
+    </row>
+    <row r="434" ht="18" customHeight="1" s="12">
+      <c r="I434" s="19" t="n"/>
+    </row>
+    <row r="435" ht="18" customHeight="1" s="12">
+      <c r="I435" s="19" t="n"/>
+    </row>
+    <row r="436" ht="18" customHeight="1" s="12">
+      <c r="I436" s="19" t="n"/>
+    </row>
+    <row r="437" ht="18" customHeight="1" s="12">
+      <c r="I437" s="19" t="n"/>
+    </row>
+    <row r="438" ht="18" customHeight="1" s="12">
+      <c r="I438" s="19" t="n"/>
+    </row>
+    <row r="439" ht="18" customHeight="1" s="12">
+      <c r="I439" s="19" t="n"/>
+    </row>
+    <row r="440" ht="18" customHeight="1" s="12">
+      <c r="I440" s="19" t="n"/>
+    </row>
+    <row r="441" ht="18" customHeight="1" s="12">
+      <c r="I441" s="19" t="n"/>
+    </row>
+    <row r="442" ht="18" customHeight="1" s="12">
+      <c r="I442" s="19" t="n"/>
+    </row>
+    <row r="443" ht="18" customHeight="1" s="12">
+      <c r="I443" s="19" t="n"/>
+    </row>
+    <row r="444" ht="18" customHeight="1" s="12">
+      <c r="I444" s="19" t="n"/>
+    </row>
+    <row r="445" ht="18" customHeight="1" s="12">
+      <c r="I445" s="19" t="n"/>
+    </row>
+    <row r="446" ht="18" customHeight="1" s="12">
+      <c r="I446" s="19" t="n"/>
+    </row>
+    <row r="447" ht="18" customHeight="1" s="12">
+      <c r="I447" s="19" t="n"/>
+    </row>
+    <row r="448" ht="18" customHeight="1" s="12">
+      <c r="I448" s="19" t="n"/>
+    </row>
+    <row r="449" ht="18" customHeight="1" s="12">
+      <c r="I449" s="19" t="n"/>
+    </row>
+    <row r="450" ht="18" customHeight="1" s="12">
+      <c r="I450" s="19" t="n"/>
+    </row>
+    <row r="451" ht="18" customHeight="1" s="12">
+      <c r="I451" s="19" t="n"/>
+    </row>
+    <row r="452" ht="18" customHeight="1" s="12">
+      <c r="I452" s="19" t="n"/>
+    </row>
+    <row r="453" ht="18" customHeight="1" s="12">
+      <c r="I453" s="19" t="n"/>
+    </row>
+    <row r="454" ht="18" customHeight="1" s="12">
+      <c r="I454" s="19" t="n"/>
+    </row>
+    <row r="455" ht="18" customHeight="1" s="12">
+      <c r="I455" s="19" t="n"/>
+    </row>
+    <row r="456" ht="18" customHeight="1" s="12">
+      <c r="I456" s="19" t="n"/>
+    </row>
+    <row r="457" ht="18" customHeight="1" s="12">
+      <c r="I457" s="19" t="n"/>
+    </row>
+    <row r="458" ht="18" customHeight="1" s="12">
+      <c r="I458" s="19" t="n"/>
+    </row>
+    <row r="459" ht="18" customHeight="1" s="12">
+      <c r="I459" s="19" t="n"/>
+    </row>
+    <row r="460" ht="18" customHeight="1" s="12">
+      <c r="I460" s="19" t="n"/>
+    </row>
+    <row r="461" ht="18" customHeight="1" s="12">
+      <c r="I461" s="19" t="n"/>
+    </row>
+    <row r="462" ht="18" customHeight="1" s="12">
+      <c r="I462" s="19" t="n"/>
+    </row>
+    <row r="463" ht="18" customHeight="1" s="12">
+      <c r="I463" s="19" t="n"/>
+    </row>
+    <row r="464" ht="18" customHeight="1" s="12">
+      <c r="I464" s="19" t="n"/>
+    </row>
+    <row r="465" ht="18" customHeight="1" s="12">
+      <c r="I465" s="19" t="n"/>
+    </row>
+    <row r="466" ht="18" customHeight="1" s="12">
+      <c r="I466" s="19" t="n"/>
+    </row>
+    <row r="467" ht="18" customHeight="1" s="12">
+      <c r="I467" s="19" t="n"/>
+    </row>
+    <row r="468" ht="18" customHeight="1" s="12">
+      <c r="I468" s="19" t="n"/>
+    </row>
+    <row r="469" ht="18" customHeight="1" s="12">
+      <c r="I469" s="19" t="n"/>
+    </row>
+    <row r="470" ht="18" customHeight="1" s="12">
+      <c r="I470" s="19" t="n"/>
+    </row>
+    <row r="471" ht="18" customHeight="1" s="12">
+      <c r="I471" s="19" t="n"/>
+    </row>
+    <row r="472" ht="18" customHeight="1" s="12">
+      <c r="I472" s="19" t="n"/>
+    </row>
+    <row r="473" ht="18" customHeight="1" s="12">
+      <c r="I473" s="19" t="n"/>
+    </row>
+    <row r="474" ht="18" customHeight="1" s="12">
+      <c r="I474" s="19" t="n"/>
+    </row>
+    <row r="475" ht="18" customHeight="1" s="12">
+      <c r="I475" s="19" t="n"/>
+    </row>
+    <row r="476" ht="18" customHeight="1" s="12">
+      <c r="I476" s="19" t="n"/>
+    </row>
+    <row r="477" ht="18" customHeight="1" s="12">
+      <c r="I477" s="19" t="n"/>
+    </row>
+    <row r="478" ht="18" customHeight="1" s="12">
+      <c r="I478" s="19" t="n"/>
+    </row>
+    <row r="479" ht="18" customHeight="1" s="12">
+      <c r="I479" s="19" t="n"/>
+    </row>
+    <row r="480" ht="18" customHeight="1" s="12">
+      <c r="I480" s="19" t="n"/>
+    </row>
+    <row r="481" ht="18" customHeight="1" s="12">
+      <c r="I481" s="19" t="n"/>
+    </row>
+    <row r="482" ht="18" customHeight="1" s="12">
+      <c r="I482" s="19" t="n"/>
+    </row>
+    <row r="483" ht="18" customHeight="1" s="12">
+      <c r="I483" s="19" t="n"/>
+    </row>
+    <row r="484" ht="18" customHeight="1" s="12">
+      <c r="I484" s="19" t="n"/>
+    </row>
+    <row r="485" ht="18" customHeight="1" s="12">
+      <c r="I485" s="19" t="n"/>
+    </row>
+    <row r="486" ht="18" customHeight="1" s="12">
+      <c r="I486" s="19" t="n"/>
+    </row>
+    <row r="487" ht="18" customHeight="1" s="12">
+      <c r="I487" s="19" t="n"/>
+    </row>
+    <row r="488" ht="18" customHeight="1" s="12">
+      <c r="I488" s="19" t="n"/>
+    </row>
+    <row r="489" ht="18" customHeight="1" s="12">
+      <c r="I489" s="19" t="n"/>
+    </row>
+    <row r="490" ht="18" customHeight="1" s="12">
+      <c r="I490" s="19" t="n"/>
+    </row>
+    <row r="491" ht="18" customHeight="1" s="12">
+      <c r="I491" s="19" t="n"/>
+    </row>
+    <row r="492" ht="18" customHeight="1" s="12">
+      <c r="I492" s="19" t="n"/>
+    </row>
+    <row r="493" ht="18" customHeight="1" s="12">
+      <c r="I493" s="19" t="n"/>
+    </row>
+    <row r="494" ht="18" customHeight="1" s="12">
+      <c r="I494" s="19" t="n"/>
+    </row>
+    <row r="495" ht="18" customHeight="1" s="12">
+      <c r="I495" s="19" t="n"/>
+    </row>
+    <row r="496" ht="18" customHeight="1" s="12">
+      <c r="I496" s="19" t="n"/>
+    </row>
+    <row r="497" ht="18" customHeight="1" s="12">
+      <c r="I497" s="19" t="n"/>
+    </row>
+    <row r="498" ht="18" customHeight="1" s="12">
+      <c r="I498" s="19" t="n"/>
+    </row>
+    <row r="499" ht="18" customHeight="1" s="12">
+      <c r="I499" s="19" t="n"/>
+    </row>
+    <row r="500" ht="18" customHeight="1" s="12">
+      <c r="I500" s="19" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="C1:D1"/>

</xml_diff>